<commit_message>
added dssp and sasa calcualtions to layer 2 (and integrated to initialpca.py, it works). For now, layer 2 is complete!
</commit_message>
<xml_diff>
--- a/494/layer2_analysis.xlsx
+++ b/494/layer2_analysis.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,103 +425,123 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S83"/>
+  <dimension ref="A1:W83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Organism</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>sequence</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>struct_type</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>index</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>pull_id</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>radius_of_gyration</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>principal_axis_1</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>principal_axis_2</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>principal_axis_3</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>axis_ratio_1</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>axis_ratio_2</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>moment_1</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>moment_2</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>moment_3</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>moment_ratio_1</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>moment_ratio_2</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>total_sasa</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>helix_fraction</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>sheet_fraction</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>coil_fraction</t>
         </is>
       </c>
     </row>
@@ -554,19 +586,19 @@
         <v>26.07182873182543</v>
       </c>
       <c r="J2" t="n">
-        <v>331.2717246896602</v>
+        <v>331.2717246896601</v>
       </c>
       <c r="K2" t="n">
-        <v>200.6963464596042</v>
+        <v>200.6963464596046</v>
       </c>
       <c r="L2" t="n">
-        <v>148.4452906887357</v>
+        <v>148.445290688736</v>
       </c>
       <c r="M2" t="n">
-        <v>1.650611635605125</v>
+        <v>1.650611635605122</v>
       </c>
       <c r="N2" t="n">
-        <v>1.351988638564696</v>
+        <v>1.351988638564695</v>
       </c>
       <c r="O2" t="n">
         <v>13824776.92599732</v>
@@ -583,6 +615,18 @@
       <c r="S2" t="n">
         <v>1.372343943791009</v>
       </c>
+      <c r="T2" t="n">
+        <v>19231.90441010254</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.3151750972762646</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.1828793774319066</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.5019455252918288</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -625,19 +669,19 @@
         <v>19.17859879704905</v>
       </c>
       <c r="J3" t="n">
-        <v>199.0190118992465</v>
+        <v>199.0190118992464</v>
       </c>
       <c r="K3" t="n">
-        <v>86.39923758051685</v>
+        <v>86.39923758051673</v>
       </c>
       <c r="L3" t="n">
-        <v>82.99213858673559</v>
+        <v>82.99213858673571</v>
       </c>
       <c r="M3" t="n">
-        <v>2.303481112478307</v>
+        <v>2.303481112478309</v>
       </c>
       <c r="N3" t="n">
-        <v>1.041053273861843</v>
+        <v>1.04105327386184</v>
       </c>
       <c r="O3" t="n">
         <v>9363896.813193027</v>
@@ -654,6 +698,18 @@
       <c r="S3" t="n">
         <v>1.659616173136139</v>
       </c>
+      <c r="T3" t="n">
+        <v>14872.73838458597</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.3084745762711865</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.2949152542372881</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.3966101694915254</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -696,19 +752,19 @@
         <v>28.19870369300713</v>
       </c>
       <c r="J4" t="n">
-        <v>470.1517222444618</v>
+        <v>470.1517222444606</v>
       </c>
       <c r="K4" t="n">
-        <v>175.0713668168456</v>
+        <v>175.0713668168454</v>
       </c>
       <c r="L4" t="n">
-        <v>151.8850082928938</v>
+        <v>151.8850082928941</v>
       </c>
       <c r="M4" t="n">
-        <v>2.685486100855774</v>
+        <v>2.685486100855771</v>
       </c>
       <c r="N4" t="n">
-        <v>1.152657321381182</v>
+        <v>1.152657321381178</v>
       </c>
       <c r="O4" t="n">
         <v>58373644.33871195</v>
@@ -725,6 +781,18 @@
       <c r="S4" t="n">
         <v>1.888789812284899</v>
       </c>
+      <c r="T4" t="n">
+        <v>34621.49545667653</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.3611442193087008</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.1561382598331347</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.4827175208581645</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -767,19 +835,19 @@
         <v>32.17200533128995</v>
       </c>
       <c r="J5" t="n">
-        <v>782.1134104793675</v>
+        <v>782.1134104793687</v>
       </c>
       <c r="K5" t="n">
-        <v>177.5613622623798</v>
+        <v>177.5613622623801</v>
       </c>
       <c r="L5" t="n">
-        <v>74.49594555745055</v>
+        <v>74.49594555745038</v>
       </c>
       <c r="M5" t="n">
-        <v>4.404750000304965</v>
+        <v>4.404750000304964</v>
       </c>
       <c r="N5" t="n">
-        <v>2.383503705251264</v>
+        <v>2.383503705251274</v>
       </c>
       <c r="O5" t="n">
         <v>46130037.53298131</v>
@@ -794,7 +862,19 @@
         <v>1.121015830634513</v>
       </c>
       <c r="S5" t="n">
-        <v>3.386911617889452</v>
+        <v>3.386911617889453</v>
+      </c>
+      <c r="T5" t="n">
+        <v>22950.34481738518</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.1693735498839907</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.3712296983758701</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.4593967517401392</v>
       </c>
     </row>
     <row r="6">
@@ -838,19 +918,19 @@
         <v>12.72266166544558</v>
       </c>
       <c r="J6" t="n">
-        <v>66.91315186518517</v>
+        <v>66.91315186518523</v>
       </c>
       <c r="K6" t="n">
-        <v>54.01376972726013</v>
+        <v>54.0137697272601</v>
       </c>
       <c r="L6" t="n">
-        <v>41.51269294972349</v>
+        <v>41.51269294972353</v>
       </c>
       <c r="M6" t="n">
-        <v>1.238816549984566</v>
+        <v>1.238816549984567</v>
       </c>
       <c r="N6" t="n">
-        <v>1.301138661196392</v>
+        <v>1.30113866119639</v>
       </c>
       <c r="O6" t="n">
         <v>1434478.286603975</v>
@@ -867,6 +947,18 @@
       <c r="S6" t="n">
         <v>1.131354128818451</v>
       </c>
+      <c r="T6" t="n">
+        <v>6030.470408868176</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.264957264957265</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.2991452991452991</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.4358974358974359</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -909,25 +1001,25 @@
         <v>13.2443724233062</v>
       </c>
       <c r="J7" t="n">
-        <v>79.27825311545408</v>
+        <v>79.27825311545412</v>
       </c>
       <c r="K7" t="n">
-        <v>55.15452303878888</v>
+        <v>55.15452303878883</v>
       </c>
       <c r="L7" t="n">
-        <v>40.4706854457061</v>
+        <v>40.47068544570612</v>
       </c>
       <c r="M7" t="n">
-        <v>1.437384438257213</v>
+        <v>1.437384438257215</v>
       </c>
       <c r="N7" t="n">
-        <v>1.362826510877411</v>
+        <v>1.362826510877409</v>
       </c>
       <c r="O7" t="n">
         <v>1798969.177441869</v>
       </c>
       <c r="P7" t="n">
-        <v>1606115.462617584</v>
+        <v>1606115.462617585</v>
       </c>
       <c r="Q7" t="n">
         <v>1278517.715761213</v>
@@ -936,7 +1028,19 @@
         <v>1.120074626832855</v>
       </c>
       <c r="S7" t="n">
-        <v>1.256232465782708</v>
+        <v>1.256232465782709</v>
+      </c>
+      <c r="T7" t="n">
+        <v>6192.284685186883</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0.291044776119403</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0.2164179104477612</v>
+      </c>
+      <c r="W7" t="n">
+        <v>0.4925373134328358</v>
       </c>
     </row>
     <row r="8">
@@ -980,16 +1084,16 @@
         <v>14.78070544523789</v>
       </c>
       <c r="J8" t="n">
-        <v>89.87502293822907</v>
+        <v>89.87502293822909</v>
       </c>
       <c r="K8" t="n">
-        <v>77.77388163266976</v>
+        <v>77.77388163266967</v>
       </c>
       <c r="L8" t="n">
-        <v>49.90903956741866</v>
+        <v>49.90903956741861</v>
       </c>
       <c r="M8" t="n">
-        <v>1.155593896710899</v>
+        <v>1.155593896710901</v>
       </c>
       <c r="N8" t="n">
         <v>1.558312528286793</v>
@@ -1009,6 +1113,18 @@
       <c r="S8" t="n">
         <v>1.092613963025785</v>
       </c>
+      <c r="T8" t="n">
+        <v>8032.405785755001</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0.3493975903614458</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0.1265060240963855</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0.5240963855421686</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1047,25 +1163,25 @@
         <v>20.66360870766868</v>
       </c>
       <c r="J9" t="n">
-        <v>359.0313815139768</v>
+        <v>359.031381513977</v>
       </c>
       <c r="K9" t="n">
-        <v>34.21319969282903</v>
+        <v>34.21319969282919</v>
       </c>
       <c r="L9" t="n">
-        <v>33.03667295921176</v>
+        <v>33.03667295921188</v>
       </c>
       <c r="M9" t="n">
-        <v>10.49394341182384</v>
+        <v>10.4939434118238</v>
       </c>
       <c r="N9" t="n">
-        <v>1.035612748749544</v>
+        <v>1.035612748749545</v>
       </c>
       <c r="O9" t="n">
-        <v>6230713.262523383</v>
+        <v>6230713.262523384</v>
       </c>
       <c r="P9" t="n">
-        <v>6209206.216761607</v>
+        <v>6209206.216761606</v>
       </c>
       <c r="Q9" t="n">
         <v>1071550.994256319</v>
@@ -1074,7 +1190,19 @@
         <v>1.003463735139561</v>
       </c>
       <c r="S9" t="n">
-        <v>5.794597037419522</v>
+        <v>5.794597037419521</v>
+      </c>
+      <c r="T9" t="n">
+        <v>9703.447466343665</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.4520547945205479</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.547945205479452</v>
       </c>
     </row>
     <row r="10">
@@ -1118,19 +1246,19 @@
         <v>14.99792187920911</v>
       </c>
       <c r="J10" t="n">
-        <v>87.22726512187731</v>
+        <v>87.22726512187738</v>
       </c>
       <c r="K10" t="n">
-        <v>81.07582068782747</v>
+        <v>81.07582068782754</v>
       </c>
       <c r="L10" t="n">
-        <v>56.3444967843257</v>
+        <v>56.34449678432582</v>
       </c>
       <c r="M10" t="n">
         <v>1.075872737171977</v>
       </c>
       <c r="N10" t="n">
-        <v>1.438930602187607</v>
+        <v>1.438930602187605</v>
       </c>
       <c r="O10" t="n">
         <v>2918294.333736918</v>
@@ -1147,6 +1275,18 @@
       <c r="S10" t="n">
         <v>1.044530460965259</v>
       </c>
+      <c r="T10" t="n">
+        <v>8069.3775937125</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0.4117647058823529</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0.1503267973856209</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.4379084967320261</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1192,25 +1332,25 @@
         <v>46.95800846976648</v>
       </c>
       <c r="K11" t="n">
-        <v>27.90937404981752</v>
+        <v>27.90937404981748</v>
       </c>
       <c r="L11" t="n">
-        <v>20.94466719355466</v>
+        <v>20.94466719355462</v>
       </c>
       <c r="M11" t="n">
-        <v>1.682517436111166</v>
+        <v>1.682517436111168</v>
       </c>
       <c r="N11" t="n">
-        <v>1.332528886322248</v>
+        <v>1.332528886322249</v>
       </c>
       <c r="O11" t="n">
         <v>403284.3926409133</v>
       </c>
       <c r="P11" t="n">
-        <v>371520.7269923738</v>
+        <v>371520.7269923737</v>
       </c>
       <c r="Q11" t="n">
-        <v>259966.3241515053</v>
+        <v>259966.3241515054</v>
       </c>
       <c r="R11" t="n">
         <v>1.085496348765466</v>
@@ -1218,6 +1358,18 @@
       <c r="S11" t="n">
         <v>1.429110975065585</v>
       </c>
+      <c r="T11" t="n">
+        <v>3320.407938281963</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0.3215686274509804</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0.1568627450980392</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0.5215686274509804</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1260,35 +1412,47 @@
         <v>17.45354776121824</v>
       </c>
       <c r="J12" t="n">
-        <v>227.1193321004083</v>
+        <v>227.119332100408</v>
       </c>
       <c r="K12" t="n">
-        <v>52.94878861958566</v>
+        <v>52.94878861958562</v>
       </c>
       <c r="L12" t="n">
-        <v>28.90534897356336</v>
+        <v>28.90534897356335</v>
       </c>
       <c r="M12" t="n">
-        <v>4.289415074859659</v>
+        <v>4.289415074859657</v>
       </c>
       <c r="N12" t="n">
         <v>1.831798974923716</v>
       </c>
       <c r="O12" t="n">
-        <v>4625832.178789714</v>
+        <v>4625832.178789713</v>
       </c>
       <c r="P12" t="n">
-        <v>4252000.555260307</v>
+        <v>4252000.55526031</v>
       </c>
       <c r="Q12" t="n">
         <v>1316709.758319346</v>
       </c>
       <c r="R12" t="n">
-        <v>1.08791899687476</v>
+        <v>1.087918996874759</v>
       </c>
       <c r="S12" t="n">
         <v>3.229261823568149</v>
       </c>
+      <c r="T12" t="n">
+        <v>8684.807135990422</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0.005921052631578948</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0.4638157894736842</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0.5302631578947369</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1331,19 +1495,19 @@
         <v>16.30416709587091</v>
       </c>
       <c r="J13" t="n">
-        <v>130.0511295818463</v>
+        <v>130.0511295818466</v>
       </c>
       <c r="K13" t="n">
-        <v>76.84263586597741</v>
+        <v>76.84263586597761</v>
       </c>
       <c r="L13" t="n">
-        <v>58.51172304299317</v>
+        <v>58.51172304299324</v>
       </c>
       <c r="M13" t="n">
         <v>1.692434520448657</v>
       </c>
       <c r="N13" t="n">
-        <v>1.31328615651115</v>
+        <v>1.313286156511152</v>
       </c>
       <c r="O13" t="n">
         <v>4637318.37870223</v>
@@ -1360,6 +1524,18 @@
       <c r="S13" t="n">
         <v>1.386815896048343</v>
       </c>
+      <c r="T13" t="n">
+        <v>9886.014588848495</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0.3201970443349754</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0.5369458128078818</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1398,19 +1574,19 @@
         <v>16.26068157528291</v>
       </c>
       <c r="J14" t="n">
-        <v>129.9500907027698</v>
+        <v>129.9500907027697</v>
       </c>
       <c r="K14" t="n">
-        <v>77.54860771061597</v>
+        <v>77.54860771061576</v>
       </c>
       <c r="L14" t="n">
-        <v>57.40678386968226</v>
+        <v>57.40678386968218</v>
       </c>
       <c r="M14" t="n">
-        <v>1.675724355847854</v>
+        <v>1.675724355847857</v>
       </c>
       <c r="N14" t="n">
-        <v>1.350861387508786</v>
+        <v>1.350861387508784</v>
       </c>
       <c r="O14" t="n">
         <v>4915114.484443315</v>
@@ -1419,7 +1595,7 @@
         <v>4438870.565022928</v>
       </c>
       <c r="Q14" t="n">
-        <v>3226771.191518639</v>
+        <v>3226771.19151864</v>
       </c>
       <c r="R14" t="n">
         <v>1.107289436004973</v>
@@ -1427,6 +1603,18 @@
       <c r="S14" t="n">
         <v>1.375638463827312</v>
       </c>
+      <c r="T14" t="n">
+        <v>9948.584164251131</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0.3398058252427185</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0.1504854368932039</v>
+      </c>
+      <c r="W14" t="n">
+        <v>0.5097087378640777</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1469,22 +1657,22 @@
         <v>17.68346873119558</v>
       </c>
       <c r="J15" t="n">
-        <v>155.8175204564329</v>
+        <v>155.817520456433</v>
       </c>
       <c r="K15" t="n">
-        <v>97.81131667809714</v>
+        <v>97.8113166780971</v>
       </c>
       <c r="L15" t="n">
-        <v>58.14148962689266</v>
+        <v>58.14148962689282</v>
       </c>
       <c r="M15" t="n">
-        <v>1.593041845753264</v>
+        <v>1.593041845753266</v>
       </c>
       <c r="N15" t="n">
-        <v>1.682298085339315</v>
+        <v>1.682298085339309</v>
       </c>
       <c r="O15" t="n">
-        <v>6191504.502626928</v>
+        <v>6191504.502626927</v>
       </c>
       <c r="P15" t="n">
         <v>5219070.87613536</v>
@@ -1498,6 +1686,18 @@
       <c r="S15" t="n">
         <v>1.368012221908365</v>
       </c>
+      <c r="T15" t="n">
+        <v>11314.61775006731</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0.4678899082568808</v>
+      </c>
+      <c r="V15" t="n">
+        <v>0.07339449541284404</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0.4587155963302753</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1540,34 +1740,46 @@
         <v>17.64488591391073</v>
       </c>
       <c r="J16" t="n">
-        <v>251.0477430191272</v>
+        <v>251.0477430191273</v>
       </c>
       <c r="K16" t="n">
-        <v>33.28550085154776</v>
+        <v>33.28550085154772</v>
       </c>
       <c r="L16" t="n">
-        <v>27.1819504631443</v>
+        <v>27.18195046314439</v>
       </c>
       <c r="M16" t="n">
-        <v>7.542255234157114</v>
+        <v>7.542255234157128</v>
       </c>
       <c r="N16" t="n">
-        <v>1.224544239261976</v>
+        <v>1.224544239261971</v>
       </c>
       <c r="O16" t="n">
         <v>2872448.62104685</v>
       </c>
       <c r="P16" t="n">
-        <v>2809337.153570839</v>
+        <v>2809337.15357084</v>
       </c>
       <c r="Q16" t="n">
-        <v>613690.7927096044</v>
+        <v>613690.7927096048</v>
       </c>
       <c r="R16" t="n">
         <v>1.022464896175168</v>
       </c>
       <c r="S16" t="n">
-        <v>4.577773020134269</v>
+        <v>4.577773020134266</v>
+      </c>
+      <c r="T16" t="n">
+        <v>6708.439949927954</v>
+      </c>
+      <c r="U16" t="n">
+        <v>0.2929292929292929</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0.1414141414141414</v>
+      </c>
+      <c r="W16" t="n">
+        <v>0.5656565656565656</v>
       </c>
     </row>
     <row r="17">
@@ -1611,25 +1823,25 @@
         <v>9.446851431609174</v>
       </c>
       <c r="J17" t="n">
-        <v>41.19881012103415</v>
+        <v>41.1988101210342</v>
       </c>
       <c r="K17" t="n">
         <v>24.20033216070482</v>
       </c>
       <c r="L17" t="n">
-        <v>23.72504265686254</v>
+        <v>23.72504265686253</v>
       </c>
       <c r="M17" t="n">
-        <v>1.702406803652494</v>
+        <v>1.702406803652496</v>
       </c>
       <c r="N17" t="n">
-        <v>1.020033241276588</v>
+        <v>1.020033241276589</v>
       </c>
       <c r="O17" t="n">
         <v>303081.3271717981</v>
       </c>
       <c r="P17" t="n">
-        <v>299505.6879083146</v>
+        <v>299505.6879083148</v>
       </c>
       <c r="Q17" t="n">
         <v>223604.5282479996</v>
@@ -1638,7 +1850,19 @@
         <v>1.011938468642966</v>
       </c>
       <c r="S17" t="n">
-        <v>1.339443750334667</v>
+        <v>1.339443750334668</v>
+      </c>
+      <c r="T17" t="n">
+        <v>3018.724070470186</v>
+      </c>
+      <c r="U17" t="n">
+        <v>0.2978723404255319</v>
+      </c>
+      <c r="V17" t="n">
+        <v>0.1276595744680851</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0.574468085106383</v>
       </c>
     </row>
     <row r="18">
@@ -1678,19 +1902,19 @@
         <v>13.10000075210337</v>
       </c>
       <c r="J18" t="n">
-        <v>93.1249790988898</v>
+        <v>93.12497909888988</v>
       </c>
       <c r="K18" t="n">
         <v>48.05548149964587</v>
       </c>
       <c r="L18" t="n">
-        <v>33.88020301791228</v>
+        <v>33.88020301791232</v>
       </c>
       <c r="M18" t="n">
-        <v>1.937863823080746</v>
+        <v>1.937863823080747</v>
       </c>
       <c r="N18" t="n">
-        <v>1.418394142273563</v>
+        <v>1.418394142273561</v>
       </c>
       <c r="O18" t="n">
         <v>1598104.758961775</v>
@@ -1699,13 +1923,25 @@
         <v>1421237.917719726</v>
       </c>
       <c r="Q18" t="n">
-        <v>937001.0523054005</v>
+        <v>937001.0523054008</v>
       </c>
       <c r="R18" t="n">
         <v>1.124445625209479</v>
       </c>
       <c r="S18" t="n">
-        <v>1.516794366690312</v>
+        <v>1.516794366690311</v>
+      </c>
+      <c r="T18" t="n">
+        <v>5979.124400097075</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" t="n">
+        <v>0.4679245283018868</v>
+      </c>
+      <c r="W18" t="n">
+        <v>0.5320754716981132</v>
       </c>
     </row>
     <row r="19">
@@ -1749,22 +1985,22 @@
         <v>10.66467748918123</v>
       </c>
       <c r="J19" t="n">
-        <v>45.86327426368655</v>
+        <v>45.86327426368658</v>
       </c>
       <c r="K19" t="n">
         <v>37.3774238775943</v>
       </c>
       <c r="L19" t="n">
-        <v>30.20616672607713</v>
+        <v>30.20616672607711</v>
       </c>
       <c r="M19" t="n">
-        <v>1.227031440526297</v>
+        <v>1.227031440526298</v>
       </c>
       <c r="N19" t="n">
-        <v>1.237410367775206</v>
+        <v>1.237410367775207</v>
       </c>
       <c r="O19" t="n">
-        <v>611334.9130290793</v>
+        <v>611334.9130290792</v>
       </c>
       <c r="P19" t="n">
         <v>560375.1524318567</v>
@@ -1776,7 +2012,19 @@
         <v>1.090938651323266</v>
       </c>
       <c r="S19" t="n">
-        <v>1.129301878938087</v>
+        <v>1.129301878938088</v>
+      </c>
+      <c r="T19" t="n">
+        <v>3974.29929979085</v>
+      </c>
+      <c r="U19" t="n">
+        <v>0.0410958904109589</v>
+      </c>
+      <c r="V19" t="n">
+        <v>0.3972602739726027</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0.5616438356164384</v>
       </c>
     </row>
     <row r="20">
@@ -1823,16 +2071,16 @@
         <v>93.69097181353729</v>
       </c>
       <c r="K20" t="n">
-        <v>60.61005141897433</v>
+        <v>60.61005141897435</v>
       </c>
       <c r="L20" t="n">
-        <v>39.05651734038802</v>
+        <v>39.05651734038801</v>
       </c>
       <c r="M20" t="n">
-        <v>1.545799246496049</v>
+        <v>1.545799246496048</v>
       </c>
       <c r="N20" t="n">
-        <v>1.551854992362516</v>
+        <v>1.551854992362517</v>
       </c>
       <c r="O20" t="n">
         <v>2145915.157753143</v>
@@ -1849,6 +2097,18 @@
       <c r="S20" t="n">
         <v>1.330949720719578</v>
       </c>
+      <c r="T20" t="n">
+        <v>6591.021097087531</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0.5804195804195804</v>
+      </c>
+      <c r="V20" t="n">
+        <v>0.06993006993006994</v>
+      </c>
+      <c r="W20" t="n">
+        <v>0.3496503496503496</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1891,16 +2151,16 @@
         <v>16.14794309694415</v>
       </c>
       <c r="J21" t="n">
-        <v>173.8043758375852</v>
+        <v>173.8043758375849</v>
       </c>
       <c r="K21" t="n">
-        <v>47.955630515462</v>
+        <v>47.95563051546201</v>
       </c>
       <c r="L21" t="n">
         <v>38.34975817012847</v>
       </c>
       <c r="M21" t="n">
-        <v>3.624274646572452</v>
+        <v>3.624274646572447</v>
       </c>
       <c r="N21" t="n">
         <v>1.250480649779319</v>
@@ -1912,13 +2172,25 @@
         <v>3292353.985779397</v>
       </c>
       <c r="Q21" t="n">
-        <v>1344813.858643399</v>
+        <v>1344813.8586434</v>
       </c>
       <c r="R21" t="n">
         <v>1.044847676886165</v>
       </c>
       <c r="S21" t="n">
-        <v>2.448185646376821</v>
+        <v>2.44818564637682</v>
+      </c>
+      <c r="T21" t="n">
+        <v>8234.218818027166</v>
+      </c>
+      <c r="U21" t="n">
+        <v>0.0218978102189781</v>
+      </c>
+      <c r="V21" t="n">
+        <v>0.4817518248175183</v>
+      </c>
+      <c r="W21" t="n">
+        <v>0.4963503649635037</v>
       </c>
     </row>
     <row r="22">
@@ -1958,19 +2230,19 @@
         <v>12.76923657910342</v>
       </c>
       <c r="J22" t="n">
-        <v>75.88123579315067</v>
+        <v>75.88123579315061</v>
       </c>
       <c r="K22" t="n">
-        <v>47.69234450223082</v>
+        <v>47.69234450223083</v>
       </c>
       <c r="L22" t="n">
-        <v>38.79536032256249</v>
+        <v>38.79536032256243</v>
       </c>
       <c r="M22" t="n">
-        <v>1.591056941845275</v>
+        <v>1.591056941845273</v>
       </c>
       <c r="N22" t="n">
-        <v>1.229331139231462</v>
+        <v>1.229331139231465</v>
       </c>
       <c r="O22" t="n">
         <v>1292793.301697541</v>
@@ -1987,6 +2259,18 @@
       <c r="S22" t="n">
         <v>1.324348994605532</v>
       </c>
+      <c r="T22" t="n">
+        <v>5984.754046632162</v>
+      </c>
+      <c r="U22" t="n">
+        <v>0.0303030303030303</v>
+      </c>
+      <c r="V22" t="n">
+        <v>0.4848484848484849</v>
+      </c>
+      <c r="W22" t="n">
+        <v>0.4848484848484849</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2029,16 +2313,16 @@
         <v>12.31487752780838</v>
       </c>
       <c r="J23" t="n">
-        <v>69.29646734924452</v>
+        <v>69.29646734924459</v>
       </c>
       <c r="K23" t="n">
-        <v>47.92862951440918</v>
+        <v>47.92862951440917</v>
       </c>
       <c r="L23" t="n">
-        <v>33.70674027899466</v>
+        <v>33.70674027899467</v>
       </c>
       <c r="M23" t="n">
-        <v>1.445826180538113</v>
+        <v>1.445826180538115</v>
       </c>
       <c r="N23" t="n">
         <v>1.421930127852716</v>
@@ -2050,7 +2334,7 @@
         <v>1007601.292254079</v>
       </c>
       <c r="Q23" t="n">
-        <v>801455.0572243374</v>
+        <v>801455.0572243377</v>
       </c>
       <c r="R23" t="n">
         <v>1.138998585851489</v>
@@ -2058,6 +2342,18 @@
       <c r="S23" t="n">
         <v>1.257214965669671</v>
       </c>
+      <c r="T23" t="n">
+        <v>5455.033557071855</v>
+      </c>
+      <c r="U23" t="n">
+        <v>0</v>
+      </c>
+      <c r="V23" t="n">
+        <v>0.5108695652173914</v>
+      </c>
+      <c r="W23" t="n">
+        <v>0.4891304347826087</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2100,13 +2396,13 @@
         <v>12.62020953198084</v>
       </c>
       <c r="J24" t="n">
-        <v>72.35863466309205</v>
+        <v>72.358634663092</v>
       </c>
       <c r="K24" t="n">
-        <v>51.6566457121852</v>
+        <v>51.65664571218518</v>
       </c>
       <c r="L24" t="n">
-        <v>35.00410788938221</v>
+        <v>35.00410788938218</v>
       </c>
       <c r="M24" t="n">
         <v>1.400761386371308</v>
@@ -2121,13 +2417,25 @@
         <v>1070087.191158924</v>
       </c>
       <c r="Q24" t="n">
-        <v>864554.6308773689</v>
+        <v>864554.6308773686</v>
       </c>
       <c r="R24" t="n">
         <v>1.156411574526579</v>
       </c>
       <c r="S24" t="n">
-        <v>1.237732299314592</v>
+        <v>1.237732299314593</v>
+      </c>
+      <c r="T24" t="n">
+        <v>5828.558164705513</v>
+      </c>
+      <c r="U24" t="n">
+        <v>0</v>
+      </c>
+      <c r="V24" t="n">
+        <v>0.5053763440860215</v>
+      </c>
+      <c r="W24" t="n">
+        <v>0.4946236559139785</v>
       </c>
     </row>
     <row r="25">
@@ -2174,32 +2482,44 @@
         <v>116.04577310716</v>
       </c>
       <c r="K25" t="n">
-        <v>92.50349221958224</v>
+        <v>92.5034922195823</v>
       </c>
       <c r="L25" t="n">
-        <v>49.8568088304232</v>
+        <v>49.85680883042318</v>
       </c>
       <c r="M25" t="n">
         <v>1.2545015363495</v>
       </c>
       <c r="N25" t="n">
-        <v>1.855383334585497</v>
+        <v>1.855383334585499</v>
       </c>
       <c r="O25" t="n">
-        <v>3745744.875452977</v>
+        <v>3745744.875452979</v>
       </c>
       <c r="P25" t="n">
         <v>2981431.840328758</v>
       </c>
       <c r="Q25" t="n">
-        <v>2559926.905636846</v>
+        <v>2559926.905636847</v>
       </c>
       <c r="R25" t="n">
-        <v>1.256357708663881</v>
+        <v>1.256357708663882</v>
       </c>
       <c r="S25" t="n">
         <v>1.164655066425442</v>
       </c>
+      <c r="T25" t="n">
+        <v>9584.061263932275</v>
+      </c>
+      <c r="U25" t="n">
+        <v>0.4213483146067415</v>
+      </c>
+      <c r="V25" t="n">
+        <v>0.0449438202247191</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0.5337078651685393</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2241,32 +2561,44 @@
         <v>107.1477875730893</v>
       </c>
       <c r="K26" t="n">
-        <v>91.25486925409778</v>
+        <v>91.25486925409773</v>
       </c>
       <c r="L26" t="n">
-        <v>42.8155520286486</v>
+        <v>42.81555202864863</v>
       </c>
       <c r="M26" t="n">
-        <v>1.174159674425021</v>
+        <v>1.174159674425022</v>
       </c>
       <c r="N26" t="n">
-        <v>2.131348655578179</v>
+        <v>2.131348655578177</v>
       </c>
       <c r="O26" t="n">
-        <v>3309901.448238791</v>
+        <v>3309901.448238792</v>
       </c>
       <c r="P26" t="n">
-        <v>2503524.299660169</v>
+        <v>2503524.299660168</v>
       </c>
       <c r="Q26" t="n">
         <v>2243262.322185122</v>
       </c>
       <c r="R26" t="n">
-        <v>1.322096793183945</v>
+        <v>1.322096793183946</v>
       </c>
       <c r="S26" t="n">
         <v>1.116019412844027</v>
       </c>
+      <c r="T26" t="n">
+        <v>8912.365731633403</v>
+      </c>
+      <c r="U26" t="n">
+        <v>0.4171779141104294</v>
+      </c>
+      <c r="V26" t="n">
+        <v>0.03680981595092025</v>
+      </c>
+      <c r="W26" t="n">
+        <v>0.5460122699386503</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2309,25 +2641,25 @@
         <v>32.68547490684087</v>
       </c>
       <c r="J27" t="n">
-        <v>971.8462138707355</v>
+        <v>971.8462138707353</v>
       </c>
       <c r="K27" t="n">
-        <v>55.38445776628908</v>
+        <v>55.38445776628927</v>
       </c>
       <c r="L27" t="n">
-        <v>41.00012119962377</v>
+        <v>41.00012119962349</v>
       </c>
       <c r="M27" t="n">
-        <v>17.5472732435465</v>
+        <v>17.54727324354644</v>
       </c>
       <c r="N27" t="n">
-        <v>1.350836440132214</v>
+        <v>1.350836440132228</v>
       </c>
       <c r="O27" t="n">
-        <v>33605501.39083415</v>
+        <v>33605501.39083416</v>
       </c>
       <c r="P27" t="n">
-        <v>33137823.07689406</v>
+        <v>33137823.07689407</v>
       </c>
       <c r="Q27" t="n">
         <v>3174140.394526855</v>
@@ -2338,6 +2670,18 @@
       <c r="S27" t="n">
         <v>10.43993615847407</v>
       </c>
+      <c r="T27" t="n">
+        <v>17048.15419353286</v>
+      </c>
+      <c r="U27" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="V27" t="n">
+        <v>0.4533333333333333</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0.5366666666666666</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2380,22 +2724,22 @@
         <v>32.62121210544897</v>
       </c>
       <c r="J28" t="n">
-        <v>965.0549536077235</v>
+        <v>965.0549536077233</v>
       </c>
       <c r="K28" t="n">
-        <v>57.3262835394783</v>
+        <v>57.32628353947836</v>
       </c>
       <c r="L28" t="n">
-        <v>42.1689251446865</v>
+        <v>42.1689251446868</v>
       </c>
       <c r="M28" t="n">
-        <v>16.83442382834968</v>
+        <v>16.83442382834966</v>
       </c>
       <c r="N28" t="n">
-        <v>1.359443792858963</v>
+        <v>1.359443792858955</v>
       </c>
       <c r="O28" t="n">
-        <v>32835790.19085748</v>
+        <v>32835790.19085747</v>
       </c>
       <c r="P28" t="n">
         <v>32360844.46495952</v>
@@ -2409,6 +2753,18 @@
       <c r="S28" t="n">
         <v>10.07762292181925</v>
       </c>
+      <c r="T28" t="n">
+        <v>17223.9099196477</v>
+      </c>
+      <c r="U28" t="n">
+        <v>0</v>
+      </c>
+      <c r="V28" t="n">
+        <v>0.5085910652920962</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.4914089347079038</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2451,34 +2807,46 @@
         <v>19.29373465679546</v>
       </c>
       <c r="J29" t="n">
-        <v>229.1262205819993</v>
+        <v>229.1262205819996</v>
       </c>
       <c r="K29" t="n">
-        <v>97.29628808780724</v>
+        <v>97.29628808780728</v>
       </c>
       <c r="L29" t="n">
-        <v>46.19619996033922</v>
+        <v>46.19619996033916</v>
       </c>
       <c r="M29" t="n">
-        <v>2.354932804581601</v>
+        <v>2.354932804581602</v>
       </c>
       <c r="N29" t="n">
-        <v>2.106153496853397</v>
+        <v>2.106153496853401</v>
       </c>
       <c r="O29" t="n">
-        <v>9393341.141259834</v>
+        <v>9393341.141259836</v>
       </c>
       <c r="P29" t="n">
-        <v>7922214.089325687</v>
+        <v>7922214.089325689</v>
       </c>
       <c r="Q29" t="n">
-        <v>4148340.580014577</v>
+        <v>4148340.580014574</v>
       </c>
       <c r="R29" t="n">
         <v>1.185696452449616</v>
       </c>
       <c r="S29" t="n">
-        <v>1.909730875881423</v>
+        <v>1.909730875881424</v>
+      </c>
+      <c r="T29" t="n">
+        <v>12913.14149280297</v>
+      </c>
+      <c r="U29" t="n">
+        <v>0.4760147601476015</v>
+      </c>
+      <c r="V29" t="n">
+        <v>0.1697416974169742</v>
+      </c>
+      <c r="W29" t="n">
+        <v>0.3542435424354243</v>
       </c>
     </row>
     <row r="30">
@@ -2522,34 +2890,46 @@
         <v>15.66571361506694</v>
       </c>
       <c r="J30" t="n">
-        <v>143.0043851293683</v>
+        <v>143.0043851293684</v>
       </c>
       <c r="K30" t="n">
-        <v>59.68171069723851</v>
+        <v>59.68171069723855</v>
       </c>
       <c r="L30" t="n">
-        <v>42.98537414397204</v>
+        <v>42.985374143972</v>
       </c>
       <c r="M30" t="n">
-        <v>2.396117394402791</v>
+        <v>2.396117394402792</v>
       </c>
       <c r="N30" t="n">
-        <v>1.388419011949157</v>
+        <v>1.388419011949159</v>
       </c>
       <c r="O30" t="n">
-        <v>2768120.142679609</v>
+        <v>2768120.142679608</v>
       </c>
       <c r="P30" t="n">
         <v>2543672.056813945</v>
       </c>
       <c r="Q30" t="n">
-        <v>1405014.988225722</v>
+        <v>1405014.988225721</v>
       </c>
       <c r="R30" t="n">
         <v>1.088237823450714</v>
       </c>
       <c r="S30" t="n">
-        <v>1.810423431871101</v>
+        <v>1.810423431871102</v>
+      </c>
+      <c r="T30" t="n">
+        <v>8062.49182707433</v>
+      </c>
+      <c r="U30" t="n">
+        <v>0.3565891472868217</v>
+      </c>
+      <c r="V30" t="n">
+        <v>0.2015503875968992</v>
+      </c>
+      <c r="W30" t="n">
+        <v>0.4418604651162791</v>
       </c>
     </row>
     <row r="31">
@@ -2589,34 +2969,46 @@
         <v>26.00366450693758</v>
       </c>
       <c r="J31" t="n">
-        <v>397.3646691570258</v>
+        <v>397.364669157026</v>
       </c>
       <c r="K31" t="n">
-        <v>173.8322729890051</v>
+        <v>173.8322729890054</v>
       </c>
       <c r="L31" t="n">
         <v>104.0963549358549</v>
       </c>
       <c r="M31" t="n">
-        <v>2.285908492850226</v>
+        <v>2.285908492850224</v>
       </c>
       <c r="N31" t="n">
-        <v>1.669917002340016</v>
+        <v>1.669917002340018</v>
       </c>
       <c r="O31" t="n">
-        <v>30140866.53210783</v>
+        <v>30140866.53210782</v>
       </c>
       <c r="P31" t="n">
         <v>26465729.05680764</v>
       </c>
       <c r="Q31" t="n">
-        <v>14655628.55972633</v>
+        <v>14655628.55972632</v>
       </c>
       <c r="R31" t="n">
         <v>1.138864017968734</v>
       </c>
       <c r="S31" t="n">
-        <v>1.805840598985667</v>
+        <v>1.805840598985668</v>
+      </c>
+      <c r="T31" t="n">
+        <v>23339.37214516848</v>
+      </c>
+      <c r="U31" t="n">
+        <v>0.6216730038022814</v>
+      </c>
+      <c r="V31" t="n">
+        <v>0</v>
+      </c>
+      <c r="W31" t="n">
+        <v>0.3783269961977186</v>
       </c>
     </row>
     <row r="32">
@@ -2660,19 +3052,19 @@
         <v>22.75958859580804</v>
       </c>
       <c r="J32" t="n">
-        <v>261.1895028031459</v>
+        <v>261.1895028031458</v>
       </c>
       <c r="K32" t="n">
         <v>188.8564043611098</v>
       </c>
       <c r="L32" t="n">
-        <v>69.00309747882812</v>
+        <v>69.00309747882829</v>
       </c>
       <c r="M32" t="n">
-        <v>1.383005801083288</v>
+        <v>1.383005801083287</v>
       </c>
       <c r="N32" t="n">
-        <v>2.736926475207227</v>
+        <v>2.736926475207221</v>
       </c>
       <c r="O32" t="n">
         <v>18947218.3876579</v>
@@ -2684,10 +3076,22 @@
         <v>10917367.71854841</v>
       </c>
       <c r="R32" t="n">
-        <v>1.369011055921966</v>
+        <v>1.369011055921965</v>
       </c>
       <c r="S32" t="n">
-        <v>1.26771189974262</v>
+        <v>1.267711899742621</v>
+      </c>
+      <c r="T32" t="n">
+        <v>19260.354128518</v>
+      </c>
+      <c r="U32" t="n">
+        <v>0.3265306122448979</v>
+      </c>
+      <c r="V32" t="n">
+        <v>0.3214285714285715</v>
+      </c>
+      <c r="W32" t="n">
+        <v>0.3520408163265306</v>
       </c>
     </row>
     <row r="33">
@@ -2731,19 +3135,19 @@
         <v>22.80140386226809</v>
       </c>
       <c r="J33" t="n">
-        <v>260.2488751117613</v>
+        <v>260.248875111761</v>
       </c>
       <c r="K33" t="n">
-        <v>190.2739903514053</v>
+        <v>190.2739903514056</v>
       </c>
       <c r="L33" t="n">
-        <v>68.50841808323969</v>
+        <v>68.5084180832397</v>
       </c>
       <c r="M33" t="n">
-        <v>1.367758539310201</v>
+        <v>1.367758539310197</v>
       </c>
       <c r="N33" t="n">
-        <v>2.77738116971577</v>
+        <v>2.777381169715774</v>
       </c>
       <c r="O33" t="n">
         <v>19663047.59944217</v>
@@ -2752,7 +3156,7 @@
         <v>14353141.66884041</v>
       </c>
       <c r="Q33" t="n">
-        <v>11304414.84325674</v>
+        <v>11304414.84325675</v>
       </c>
       <c r="R33" t="n">
         <v>1.369947294683865</v>
@@ -2760,6 +3164,18 @@
       <c r="S33" t="n">
         <v>1.269693466478035</v>
       </c>
+      <c r="T33" t="n">
+        <v>18139.89244976177</v>
+      </c>
+      <c r="U33" t="n">
+        <v>0.3425692695214106</v>
+      </c>
+      <c r="V33" t="n">
+        <v>0.309823677581864</v>
+      </c>
+      <c r="W33" t="n">
+        <v>0.3476070528967254</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2802,16 +3218,16 @@
         <v>13.69280672555647</v>
       </c>
       <c r="J34" t="n">
-        <v>88.07758655463374</v>
+        <v>88.07758655463381</v>
       </c>
       <c r="K34" t="n">
-        <v>53.9110847239969</v>
+        <v>53.91108472399688</v>
       </c>
       <c r="L34" t="n">
-        <v>44.03642837067064</v>
+        <v>44.03642837067063</v>
       </c>
       <c r="M34" t="n">
-        <v>1.633756527169795</v>
+        <v>1.633756527169796</v>
       </c>
       <c r="N34" t="n">
         <v>1.224238357166655</v>
@@ -2823,13 +3239,25 @@
         <v>1714023.046152871</v>
       </c>
       <c r="Q34" t="n">
-        <v>1294879.165997903</v>
+        <v>1294879.165997902</v>
       </c>
       <c r="R34" t="n">
         <v>1.085330130357113</v>
       </c>
       <c r="S34" t="n">
-        <v>1.323693431141085</v>
+        <v>1.323693431141086</v>
+      </c>
+      <c r="T34" t="n">
+        <v>6920.221794945333</v>
+      </c>
+      <c r="U34" t="n">
+        <v>0.4031007751937984</v>
+      </c>
+      <c r="V34" t="n">
+        <v>0.2635658914728682</v>
+      </c>
+      <c r="W34" t="n">
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="35">
@@ -2873,25 +3301,25 @@
         <v>13.63636899560306</v>
       </c>
       <c r="J35" t="n">
-        <v>86.75997623578209</v>
+        <v>86.75997623578203</v>
       </c>
       <c r="K35" t="n">
-        <v>56.14790045161818</v>
+        <v>56.14790045161812</v>
       </c>
       <c r="L35" t="n">
-        <v>42.71937633943344</v>
+        <v>42.71937633943343</v>
       </c>
       <c r="M35" t="n">
-        <v>1.545204282581178</v>
+        <v>1.545204282581179</v>
       </c>
       <c r="N35" t="n">
-        <v>1.314342700265245</v>
+        <v>1.314342700265244</v>
       </c>
       <c r="O35" t="n">
         <v>1688057.778983845</v>
       </c>
       <c r="P35" t="n">
-        <v>1530324.270776347</v>
+        <v>1530324.270776348</v>
       </c>
       <c r="Q35" t="n">
         <v>1166120.90068483</v>
@@ -2902,6 +3330,18 @@
       <c r="S35" t="n">
         <v>1.312320420530694</v>
       </c>
+      <c r="T35" t="n">
+        <v>6817.952902177864</v>
+      </c>
+      <c r="U35" t="n">
+        <v>0.3539823008849557</v>
+      </c>
+      <c r="V35" t="n">
+        <v>0.2743362831858407</v>
+      </c>
+      <c r="W35" t="n">
+        <v>0.3716814159292036</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2944,16 +3384,16 @@
         <v>15.78310621579051</v>
       </c>
       <c r="J36" t="n">
-        <v>116.8951959220535</v>
+        <v>116.8951959220534</v>
       </c>
       <c r="K36" t="n">
-        <v>83.69368535738676</v>
+        <v>83.69368535738674</v>
       </c>
       <c r="L36" t="n">
-        <v>47.48703709727601</v>
+        <v>47.48703709727599</v>
       </c>
       <c r="M36" t="n">
-        <v>1.396702695345419</v>
+        <v>1.396702695345418</v>
       </c>
       <c r="N36" t="n">
         <v>1.762453302486368</v>
@@ -2968,11 +3408,23 @@
         <v>2552613.628915533</v>
       </c>
       <c r="R36" t="n">
-        <v>1.217625880683155</v>
+        <v>1.217625880683154</v>
       </c>
       <c r="S36" t="n">
         <v>1.257739104247261</v>
       </c>
+      <c r="T36" t="n">
+        <v>9374.940220923681</v>
+      </c>
+      <c r="U36" t="n">
+        <v>0.6777777777777778</v>
+      </c>
+      <c r="V36" t="n">
+        <v>0.03333333333333333</v>
+      </c>
+      <c r="W36" t="n">
+        <v>0.2888888888888889</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3015,25 +3467,25 @@
         <v>26.3566018632606</v>
       </c>
       <c r="J37" t="n">
-        <v>305.0021578223521</v>
+        <v>305.0021578223526</v>
       </c>
       <c r="K37" t="n">
-        <v>275.6774187318806</v>
+        <v>275.6774187318808</v>
       </c>
       <c r="L37" t="n">
-        <v>113.0607919992102</v>
+        <v>113.0607919992108</v>
       </c>
       <c r="M37" t="n">
-        <v>1.106373380980443</v>
+        <v>1.106373380980444</v>
       </c>
       <c r="N37" t="n">
-        <v>2.438311406254842</v>
+        <v>2.438311406254832</v>
       </c>
       <c r="O37" t="n">
-        <v>37528807.00099394</v>
+        <v>37528807.00099395</v>
       </c>
       <c r="P37" t="n">
-        <v>27012628.99314202</v>
+        <v>27012628.99314201</v>
       </c>
       <c r="Q37" t="n">
         <v>25123781.84201265</v>
@@ -3044,6 +3496,18 @@
       <c r="S37" t="n">
         <v>1.075181641164022</v>
       </c>
+      <c r="T37" t="n">
+        <v>27591.6573504273</v>
+      </c>
+      <c r="U37" t="n">
+        <v>0.4162679425837321</v>
+      </c>
+      <c r="V37" t="n">
+        <v>0.1578947368421053</v>
+      </c>
+      <c r="W37" t="n">
+        <v>0.4258373205741627</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3086,19 +3550,19 @@
         <v>16.05338435760597</v>
       </c>
       <c r="J38" t="n">
-        <v>139.684713457943</v>
+        <v>139.6847134579432</v>
       </c>
       <c r="K38" t="n">
-        <v>67.67842157284288</v>
+        <v>67.67842157284296</v>
       </c>
       <c r="L38" t="n">
-        <v>49.11758333904554</v>
+        <v>49.11758333904555</v>
       </c>
       <c r="M38" t="n">
         <v>2.063947565733327</v>
       </c>
       <c r="N38" t="n">
-        <v>1.377885819537921</v>
+        <v>1.377885819537922</v>
       </c>
       <c r="O38" t="n">
         <v>4058549.14204949</v>
@@ -3107,13 +3571,25 @@
         <v>3689681.015240676</v>
       </c>
       <c r="Q38" t="n">
-        <v>2273935.839527467</v>
+        <v>2273935.839527465</v>
       </c>
       <c r="R38" t="n">
         <v>1.099972904238919</v>
       </c>
       <c r="S38" t="n">
-        <v>1.622596799392285</v>
+        <v>1.622596799392286</v>
+      </c>
+      <c r="T38" t="n">
+        <v>9189.052096251156</v>
+      </c>
+      <c r="U38" t="n">
+        <v>0.3212435233160622</v>
+      </c>
+      <c r="V38" t="n">
+        <v>0.1865284974093264</v>
+      </c>
+      <c r="W38" t="n">
+        <v>0.4922279792746114</v>
       </c>
     </row>
     <row r="39">
@@ -3163,16 +3639,16 @@
         <v>85.80813160259319</v>
       </c>
       <c r="L39" t="n">
-        <v>49.21252307594495</v>
+        <v>49.21252307594506</v>
       </c>
       <c r="M39" t="n">
         <v>1.836471610171838</v>
       </c>
       <c r="N39" t="n">
-        <v>1.743623903821671</v>
+        <v>1.743623903821667</v>
       </c>
       <c r="O39" t="n">
-        <v>5396555.438234123</v>
+        <v>5396555.438234124</v>
       </c>
       <c r="P39" t="n">
         <v>4579717.318773062</v>
@@ -3186,6 +3662,18 @@
       <c r="S39" t="n">
         <v>1.529617814302956</v>
       </c>
+      <c r="T39" t="n">
+        <v>10732.536621874</v>
+      </c>
+      <c r="U39" t="n">
+        <v>0.3253588516746411</v>
+      </c>
+      <c r="V39" t="n">
+        <v>0.1866028708133971</v>
+      </c>
+      <c r="W39" t="n">
+        <v>0.4880382775119617</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3228,19 +3716,19 @@
         <v>14.52623153908031</v>
       </c>
       <c r="J40" t="n">
-        <v>112.7628892205886</v>
+        <v>112.7628892205887</v>
       </c>
       <c r="K40" t="n">
-        <v>53.58205648037577</v>
+        <v>53.58205648037579</v>
       </c>
       <c r="L40" t="n">
-        <v>40.9556183332525</v>
+        <v>40.95561833325242</v>
       </c>
       <c r="M40" t="n">
-        <v>2.104489760707255</v>
+        <v>2.104489760707256</v>
       </c>
       <c r="N40" t="n">
-        <v>1.308295629781071</v>
+        <v>1.308295629781074</v>
       </c>
       <c r="O40" t="n">
         <v>2594207.844208319</v>
@@ -3257,6 +3745,18 @@
       <c r="S40" t="n">
         <v>1.636734187472904</v>
       </c>
+      <c r="T40" t="n">
+        <v>7148.675862592751</v>
+      </c>
+      <c r="U40" t="n">
+        <v>0.352112676056338</v>
+      </c>
+      <c r="V40" t="n">
+        <v>0.1830985915492958</v>
+      </c>
+      <c r="W40" t="n">
+        <v>0.4647887323943662</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3299,19 +3799,19 @@
         <v>35.36257834381378</v>
       </c>
       <c r="J41" t="n">
-        <v>720.7789469691095</v>
+        <v>720.7789469691093</v>
       </c>
       <c r="K41" t="n">
-        <v>367.6698531017863</v>
+        <v>367.6698531017856</v>
       </c>
       <c r="L41" t="n">
-        <v>162.5146905334817</v>
+        <v>162.5146905334816</v>
       </c>
       <c r="M41" t="n">
-        <v>1.960397190273764</v>
+        <v>1.960397190273767</v>
       </c>
       <c r="N41" t="n">
-        <v>2.262379184889983</v>
+        <v>2.262379184889981</v>
       </c>
       <c r="O41" t="n">
         <v>40089352.05075736</v>
@@ -3328,6 +3828,18 @@
       <c r="S41" t="n">
         <v>1.671786984394734</v>
       </c>
+      <c r="T41" t="n">
+        <v>35154.15727768082</v>
+      </c>
+      <c r="U41" t="n">
+        <v>0.1552631578947369</v>
+      </c>
+      <c r="V41" t="n">
+        <v>0.08947368421052632</v>
+      </c>
+      <c r="W41" t="n">
+        <v>0.7552631578947369</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3370,19 +3882,19 @@
         <v>24.33592112517048</v>
       </c>
       <c r="J42" t="n">
-        <v>318.2740164054542</v>
+        <v>318.2740164054541</v>
       </c>
       <c r="K42" t="n">
-        <v>187.7031650652895</v>
+        <v>187.7031650652898</v>
       </c>
       <c r="L42" t="n">
-        <v>88.78095303522149</v>
+        <v>88.78095303522132</v>
       </c>
       <c r="M42" t="n">
-        <v>1.695624132362114</v>
+        <v>1.695624132362111</v>
       </c>
       <c r="N42" t="n">
-        <v>2.114227868119677</v>
+        <v>2.114227868119685</v>
       </c>
       <c r="O42" t="n">
         <v>13243108.21211964</v>
@@ -3391,7 +3903,7 @@
         <v>10665248.84419503</v>
       </c>
       <c r="Q42" t="n">
-        <v>7277940.243162015</v>
+        <v>7277940.243162017</v>
       </c>
       <c r="R42" t="n">
         <v>1.241706443570486</v>
@@ -3399,6 +3911,18 @@
       <c r="S42" t="n">
         <v>1.465421326345123</v>
       </c>
+      <c r="T42" t="n">
+        <v>18860.19465162126</v>
+      </c>
+      <c r="U42" t="n">
+        <v>0.2213438735177866</v>
+      </c>
+      <c r="V42" t="n">
+        <v>0.1778656126482213</v>
+      </c>
+      <c r="W42" t="n">
+        <v>0.6007905138339921</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3444,16 +3968,16 @@
         <v>330.7414750735209</v>
       </c>
       <c r="K43" t="n">
-        <v>114.4441701113891</v>
+        <v>114.444170111389</v>
       </c>
       <c r="L43" t="n">
-        <v>57.25929912862778</v>
+        <v>57.25929912862762</v>
       </c>
       <c r="M43" t="n">
-        <v>2.889980981570389</v>
+        <v>2.889980981570393</v>
       </c>
       <c r="N43" t="n">
-        <v>1.998700156184252</v>
+        <v>1.998700156184254</v>
       </c>
       <c r="O43" t="n">
         <v>11065857.56447235</v>
@@ -3462,13 +3986,25 @@
         <v>9630192.838040654</v>
       </c>
       <c r="Q43" t="n">
-        <v>4259745.607651558</v>
+        <v>4259745.607651554</v>
       </c>
       <c r="R43" t="n">
         <v>1.149079540833349</v>
       </c>
       <c r="S43" t="n">
-        <v>2.260743651156643</v>
+        <v>2.260743651156644</v>
+      </c>
+      <c r="T43" t="n">
+        <v>14205.1224032963</v>
+      </c>
+      <c r="U43" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="V43" t="n">
+        <v>0.1833333333333333</v>
+      </c>
+      <c r="W43" t="n">
+        <v>0.5166666666666667</v>
       </c>
     </row>
     <row r="44">
@@ -3512,19 +4048,19 @@
         <v>16.78968194755778</v>
       </c>
       <c r="J44" t="n">
-        <v>183.6760033120122</v>
+        <v>183.6760033120124</v>
       </c>
       <c r="K44" t="n">
-        <v>54.317680627896</v>
+        <v>54.31768062789585</v>
       </c>
       <c r="L44" t="n">
-        <v>43.40368903694139</v>
+        <v>43.40368903694144</v>
       </c>
       <c r="M44" t="n">
-        <v>3.381514107170501</v>
+        <v>3.381514107170515</v>
       </c>
       <c r="N44" t="n">
-        <v>1.251453086894655</v>
+        <v>1.25145308689465</v>
       </c>
       <c r="O44" t="n">
         <v>4061922.765786008</v>
@@ -3539,7 +4075,19 @@
         <v>1.048718065987322</v>
       </c>
       <c r="S44" t="n">
-        <v>2.322511892335138</v>
+        <v>2.322511892335137</v>
+      </c>
+      <c r="T44" t="n">
+        <v>8665.181417466503</v>
+      </c>
+      <c r="U44" t="n">
+        <v>0.6402439024390244</v>
+      </c>
+      <c r="V44" t="n">
+        <v>0.07317073170731707</v>
+      </c>
+      <c r="W44" t="n">
+        <v>0.2865853658536585</v>
       </c>
     </row>
     <row r="45">
@@ -3583,19 +4131,19 @@
         <v>13.98214462110945</v>
       </c>
       <c r="J45" t="n">
-        <v>90.24212835629041</v>
+        <v>90.24212835629056</v>
       </c>
       <c r="K45" t="n">
         <v>63.01924720999455</v>
       </c>
       <c r="L45" t="n">
-        <v>41.92890536144371</v>
+        <v>41.92890536144375</v>
       </c>
       <c r="M45" t="n">
-        <v>1.431977250626035</v>
+        <v>1.431977250626037</v>
       </c>
       <c r="N45" t="n">
-        <v>1.503002443463376</v>
+        <v>1.503002443463375</v>
       </c>
       <c r="O45" t="n">
         <v>1993769.294435629</v>
@@ -3612,6 +4160,18 @@
       <c r="S45" t="n">
         <v>1.260374775481222</v>
       </c>
+      <c r="T45" t="n">
+        <v>7005.440785573033</v>
+      </c>
+      <c r="U45" t="n">
+        <v>0.265625</v>
+      </c>
+      <c r="V45" t="n">
+        <v>0.3203125</v>
+      </c>
+      <c r="W45" t="n">
+        <v>0.4140625</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3657,16 +4217,16 @@
         <v>103.1373902549663</v>
       </c>
       <c r="K46" t="n">
-        <v>44.23847904438629</v>
+        <v>44.23847904438624</v>
       </c>
       <c r="L46" t="n">
         <v>36.57182174192813</v>
       </c>
       <c r="M46" t="n">
-        <v>2.331395483815895</v>
+        <v>2.331395483815897</v>
       </c>
       <c r="N46" t="n">
-        <v>1.209632906901891</v>
+        <v>1.209632906901889</v>
       </c>
       <c r="O46" t="n">
         <v>1988837.079281489</v>
@@ -3683,6 +4243,18 @@
       <c r="S46" t="n">
         <v>1.740150809928003</v>
       </c>
+      <c r="T46" t="n">
+        <v>6409.688484362101</v>
+      </c>
+      <c r="U46" t="n">
+        <v>0.40625</v>
+      </c>
+      <c r="V46" t="n">
+        <v>0.1015625</v>
+      </c>
+      <c r="W46" t="n">
+        <v>0.4921875</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3725,19 +4297,19 @@
         <v>22.61210337468428</v>
       </c>
       <c r="J47" t="n">
-        <v>324.357395777229</v>
+        <v>324.3573957772289</v>
       </c>
       <c r="K47" t="n">
-        <v>107.2589186787522</v>
+        <v>107.2589186787519</v>
       </c>
       <c r="L47" t="n">
-        <v>78.862258082902</v>
+        <v>78.86225808290169</v>
       </c>
       <c r="M47" t="n">
-        <v>3.024059908236645</v>
+        <v>3.024059908236652</v>
       </c>
       <c r="N47" t="n">
-        <v>1.360079222763301</v>
+        <v>1.360079222763302</v>
       </c>
       <c r="O47" t="n">
         <v>17461955.53963</v>
@@ -3754,6 +4326,18 @@
       <c r="S47" t="n">
         <v>2.164415843756435</v>
       </c>
+      <c r="T47" t="n">
+        <v>17133.65549496524</v>
+      </c>
+      <c r="U47" t="n">
+        <v>0.6125</v>
+      </c>
+      <c r="V47" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="W47" t="n">
+        <v>0.3725</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3796,22 +4380,22 @@
         <v>13.76898045854512</v>
       </c>
       <c r="J48" t="n">
-        <v>93.34627803637802</v>
+        <v>93.346278036378</v>
       </c>
       <c r="K48" t="n">
-        <v>53.65684289815947</v>
+        <v>53.65684289815938</v>
       </c>
       <c r="L48" t="n">
         <v>43.19384829762701</v>
       </c>
       <c r="M48" t="n">
-        <v>1.739690093462058</v>
+        <v>1.73969009346206</v>
       </c>
       <c r="N48" t="n">
-        <v>1.24223344325417</v>
+        <v>1.242233443254168</v>
       </c>
       <c r="O48" t="n">
-        <v>2073790.582118271</v>
+        <v>2073790.58211827</v>
       </c>
       <c r="P48" t="n">
         <v>1931218.007767265</v>
@@ -3825,6 +4409,18 @@
       <c r="S48" t="n">
         <v>1.413884346895441</v>
       </c>
+      <c r="T48" t="n">
+        <v>6760.990015426727</v>
+      </c>
+      <c r="U48" t="n">
+        <v>0.5547445255474452</v>
+      </c>
+      <c r="V48" t="n">
+        <v>0.0583941605839416</v>
+      </c>
+      <c r="W48" t="n">
+        <v>0.3868613138686132</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3867,19 +4463,19 @@
         <v>19.97436242110372</v>
       </c>
       <c r="J49" t="n">
-        <v>208.8865964561399</v>
+        <v>208.8865964561398</v>
       </c>
       <c r="K49" t="n">
         <v>107.317947995299</v>
       </c>
       <c r="L49" t="n">
-        <v>81.81392885194137</v>
+        <v>81.81392885194111</v>
       </c>
       <c r="M49" t="n">
-        <v>1.94642741832233</v>
+        <v>1.946427418322329</v>
       </c>
       <c r="N49" t="n">
-        <v>1.311731993576696</v>
+        <v>1.3117319935767</v>
       </c>
       <c r="O49" t="n">
         <v>10705487.14620506</v>
@@ -3888,13 +4484,25 @@
         <v>9849387.733521545</v>
       </c>
       <c r="Q49" t="n">
-        <v>6399616.826065045</v>
+        <v>6399616.826065044</v>
       </c>
       <c r="R49" t="n">
         <v>1.086919048761767</v>
       </c>
       <c r="S49" t="n">
-        <v>1.539058978250995</v>
+        <v>1.539058978250996</v>
+      </c>
+      <c r="T49" t="n">
+        <v>15938.65733286129</v>
+      </c>
+      <c r="U49" t="n">
+        <v>0.2761904761904762</v>
+      </c>
+      <c r="V49" t="n">
+        <v>0.3492063492063492</v>
+      </c>
+      <c r="W49" t="n">
+        <v>0.3746031746031746</v>
       </c>
     </row>
     <row r="50">
@@ -3938,19 +4546,19 @@
         <v>20.78900601566003</v>
       </c>
       <c r="J50" t="n">
-        <v>272.3923545408315</v>
+        <v>272.3923545408318</v>
       </c>
       <c r="K50" t="n">
-        <v>116.95196641812</v>
+        <v>116.9519664181199</v>
       </c>
       <c r="L50" t="n">
-        <v>43.02178745554333</v>
+        <v>43.0217874555433</v>
       </c>
       <c r="M50" t="n">
-        <v>2.329095977463003</v>
+        <v>2.329095977463008</v>
       </c>
       <c r="N50" t="n">
-        <v>2.718435781845945</v>
+        <v>2.718435781845944</v>
       </c>
       <c r="O50" t="n">
         <v>9353337.851389566</v>
@@ -3967,6 +4575,18 @@
       <c r="S50" t="n">
         <v>1.973982925733489</v>
       </c>
+      <c r="T50" t="n">
+        <v>12116.64616485599</v>
+      </c>
+      <c r="U50" t="n">
+        <v>0.3628691983122363</v>
+      </c>
+      <c r="V50" t="n">
+        <v>0.1772151898734177</v>
+      </c>
+      <c r="W50" t="n">
+        <v>0.459915611814346</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4012,25 +4632,25 @@
         <v>117.9413200760066</v>
       </c>
       <c r="K51" t="n">
-        <v>72.0064784801317</v>
+        <v>72.00647848013156</v>
       </c>
       <c r="L51" t="n">
-        <v>61.31840707824568</v>
+        <v>61.31840707824566</v>
       </c>
       <c r="M51" t="n">
-        <v>1.637926511133986</v>
+        <v>1.63792651113399</v>
       </c>
       <c r="N51" t="n">
-        <v>1.174304452955659</v>
+        <v>1.174304452955657</v>
       </c>
       <c r="O51" t="n">
         <v>4571464.52168483</v>
       </c>
       <c r="P51" t="n">
-        <v>4359445.61108726</v>
+        <v>4359445.611087261</v>
       </c>
       <c r="Q51" t="n">
-        <v>3211024.757133762</v>
+        <v>3211024.757133763</v>
       </c>
       <c r="R51" t="n">
         <v>1.048634374531098</v>
@@ -4038,6 +4658,18 @@
       <c r="S51" t="n">
         <v>1.357649330296228</v>
       </c>
+      <c r="T51" t="n">
+        <v>8848.900650340885</v>
+      </c>
+      <c r="U51" t="n">
+        <v>0.2704081632653061</v>
+      </c>
+      <c r="V51" t="n">
+        <v>0.2142857142857143</v>
+      </c>
+      <c r="W51" t="n">
+        <v>0.5153061224489796</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4080,19 +4712,19 @@
         <v>22.29120847660255</v>
       </c>
       <c r="J52" t="n">
-        <v>235.752659480885</v>
+        <v>235.7526594808851</v>
       </c>
       <c r="K52" t="n">
-        <v>158.340711637694</v>
+        <v>158.3407116376939</v>
       </c>
       <c r="L52" t="n">
-        <v>104.2762026520008</v>
+        <v>104.2762026520009</v>
       </c>
       <c r="M52" t="n">
-        <v>1.488894782917993</v>
+        <v>1.488894782917996</v>
       </c>
       <c r="N52" t="n">
-        <v>1.518474087190553</v>
+        <v>1.51847408719055</v>
       </c>
       <c r="O52" t="n">
         <v>20818889.97729903</v>
@@ -4109,6 +4741,18 @@
       <c r="S52" t="n">
         <v>1.290448935131623</v>
       </c>
+      <c r="T52" t="n">
+        <v>19265.35991668186</v>
+      </c>
+      <c r="U52" t="n">
+        <v>0.4338919925512104</v>
+      </c>
+      <c r="V52" t="n">
+        <v>0.111731843575419</v>
+      </c>
+      <c r="W52" t="n">
+        <v>0.4543761638733706</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4151,19 +4795,19 @@
         <v>20.98584952439502</v>
       </c>
       <c r="J53" t="n">
-        <v>202.722649044361</v>
+        <v>202.7226490443609</v>
       </c>
       <c r="K53" t="n">
-        <v>152.7836865296826</v>
+        <v>152.7836865296824</v>
       </c>
       <c r="L53" t="n">
-        <v>84.28489719265355</v>
+        <v>84.28489719265383</v>
       </c>
       <c r="M53" t="n">
-        <v>1.326860567701882</v>
+        <v>1.326860567701883</v>
       </c>
       <c r="N53" t="n">
-        <v>1.812705379238447</v>
+        <v>1.812705379238439</v>
       </c>
       <c r="O53" t="n">
         <v>15350594.29916175</v>
@@ -4180,6 +4824,18 @@
       <c r="S53" t="n">
         <v>1.211964750658296</v>
       </c>
+      <c r="T53" t="n">
+        <v>16969.49448869975</v>
+      </c>
+      <c r="U53" t="n">
+        <v>0.423963133640553</v>
+      </c>
+      <c r="V53" t="n">
+        <v>0.1658986175115207</v>
+      </c>
+      <c r="W53" t="n">
+        <v>0.4101382488479263</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4222,22 +4878,22 @@
         <v>21.2450901060281</v>
       </c>
       <c r="J54" t="n">
-        <v>175.7188624078646</v>
+        <v>175.7188624078643</v>
       </c>
       <c r="K54" t="n">
-        <v>171.8866322806966</v>
+        <v>171.8866322806968</v>
       </c>
       <c r="L54" t="n">
-        <v>103.4635858552077</v>
+        <v>103.4635858552078</v>
       </c>
       <c r="M54" t="n">
-        <v>1.022295102744871</v>
+        <v>1.022295102744868</v>
       </c>
       <c r="N54" t="n">
-        <v>1.661324908274914</v>
+        <v>1.661324908274915</v>
       </c>
       <c r="O54" t="n">
-        <v>16729278.84363357</v>
+        <v>16729278.84363358</v>
       </c>
       <c r="P54" t="n">
         <v>13433477.08761454</v>
@@ -4251,6 +4907,18 @@
       <c r="S54" t="n">
         <v>1.013019379487288</v>
       </c>
+      <c r="T54" t="n">
+        <v>18187.2350424355</v>
+      </c>
+      <c r="U54" t="n">
+        <v>0.3983572895277208</v>
+      </c>
+      <c r="V54" t="n">
+        <v>0.1437371663244353</v>
+      </c>
+      <c r="W54" t="n">
+        <v>0.457905544147844</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4293,25 +4961,25 @@
         <v>14.28076879567328</v>
       </c>
       <c r="J55" t="n">
-        <v>92.39482183239598</v>
+        <v>92.39482183239599</v>
       </c>
       <c r="K55" t="n">
-        <v>66.61710335705241</v>
+        <v>66.61710335705236</v>
       </c>
       <c r="L55" t="n">
-        <v>45.04204473350979</v>
+        <v>45.04204473350983</v>
       </c>
       <c r="M55" t="n">
-        <v>1.386953457540489</v>
+        <v>1.38695345754049</v>
       </c>
       <c r="N55" t="n">
-        <v>1.478998206035959</v>
+        <v>1.478998206035957</v>
       </c>
       <c r="O55" t="n">
-        <v>2638338.502459755</v>
+        <v>2638338.502459754</v>
       </c>
       <c r="P55" t="n">
-        <v>2283754.308646132</v>
+        <v>2283754.308646131</v>
       </c>
       <c r="Q55" t="n">
         <v>1856296.504728999</v>
@@ -4322,6 +4990,18 @@
       <c r="S55" t="n">
         <v>1.230274529326627</v>
       </c>
+      <c r="T55" t="n">
+        <v>7181.44841851191</v>
+      </c>
+      <c r="U55" t="n">
+        <v>0.4203821656050956</v>
+      </c>
+      <c r="V55" t="n">
+        <v>0.1656050955414013</v>
+      </c>
+      <c r="W55" t="n">
+        <v>0.4140127388535032</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4367,19 +5047,19 @@
         <v>117.3577409689647</v>
       </c>
       <c r="K56" t="n">
-        <v>68.73463338200634</v>
+        <v>68.73463338200636</v>
       </c>
       <c r="L56" t="n">
-        <v>51.28150493293101</v>
+        <v>51.28150493293106</v>
       </c>
       <c r="M56" t="n">
-        <v>1.707403316123414</v>
+        <v>1.707403316123413</v>
       </c>
       <c r="N56" t="n">
-        <v>1.340339630669996</v>
+        <v>1.340339630669995</v>
       </c>
       <c r="O56" t="n">
-        <v>3155907.313131475</v>
+        <v>3155907.313131476</v>
       </c>
       <c r="P56" t="n">
         <v>2856810.932863906</v>
@@ -4393,6 +5073,18 @@
       <c r="S56" t="n">
         <v>1.400148750320988</v>
       </c>
+      <c r="T56" t="n">
+        <v>8892.353374940834</v>
+      </c>
+      <c r="U56" t="n">
+        <v>0.3439490445859872</v>
+      </c>
+      <c r="V56" t="n">
+        <v>0.3312101910828025</v>
+      </c>
+      <c r="W56" t="n">
+        <v>0.3248407643312102</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4435,28 +5127,28 @@
         <v>17.89888139315902</v>
       </c>
       <c r="J57" t="n">
-        <v>147.5710386075176</v>
+        <v>147.5710386075177</v>
       </c>
       <c r="K57" t="n">
-        <v>94.01054061775339</v>
+        <v>94.01054061775342</v>
       </c>
       <c r="L57" t="n">
-        <v>77.80019842208587</v>
+        <v>77.80019842208593</v>
       </c>
       <c r="M57" t="n">
-        <v>1.569728645722197</v>
+        <v>1.569728645722198</v>
       </c>
       <c r="N57" t="n">
-        <v>1.20835862278554</v>
+        <v>1.208358622785539</v>
       </c>
       <c r="O57" t="n">
         <v>6702471.214588236</v>
       </c>
       <c r="P57" t="n">
-        <v>6243151.999699802</v>
+        <v>6243151.999699801</v>
       </c>
       <c r="Q57" t="n">
-        <v>4760097.144044517</v>
+        <v>4760097.144044518</v>
       </c>
       <c r="R57" t="n">
         <v>1.073571685409953</v>
@@ -4464,6 +5156,18 @@
       <c r="S57" t="n">
         <v>1.311559787705336</v>
       </c>
+      <c r="T57" t="n">
+        <v>12697.33742915262</v>
+      </c>
+      <c r="U57" t="n">
+        <v>0.3161764705882353</v>
+      </c>
+      <c r="V57" t="n">
+        <v>0.2683823529411765</v>
+      </c>
+      <c r="W57" t="n">
+        <v>0.4154411764705883</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4506,34 +5210,46 @@
         <v>17.61581924348128</v>
       </c>
       <c r="J58" t="n">
-        <v>159.3610546156441</v>
+        <v>159.3610546156437</v>
       </c>
       <c r="K58" t="n">
-        <v>83.7350550474071</v>
+        <v>83.7350550474068</v>
       </c>
       <c r="L58" t="n">
         <v>63.44441752456009</v>
       </c>
       <c r="M58" t="n">
-        <v>1.903158175813235</v>
+        <v>1.903158175813237</v>
       </c>
       <c r="N58" t="n">
-        <v>1.3198175397385</v>
+        <v>1.319817539738496</v>
       </c>
       <c r="O58" t="n">
-        <v>6207806.306386341</v>
+        <v>6207806.306386343</v>
       </c>
       <c r="P58" t="n">
-        <v>5714301.137816863</v>
+        <v>5714301.137816862</v>
       </c>
       <c r="Q58" t="n">
-        <v>3751141.004855778</v>
+        <v>3751141.004855775</v>
       </c>
       <c r="R58" t="n">
-        <v>1.086363171395272</v>
+        <v>1.086363171395273</v>
       </c>
       <c r="S58" t="n">
-        <v>1.523350130112361</v>
+        <v>1.523350130112362</v>
+      </c>
+      <c r="T58" t="n">
+        <v>11170.54696509023</v>
+      </c>
+      <c r="U58" t="n">
+        <v>0.3302325581395349</v>
+      </c>
+      <c r="V58" t="n">
+        <v>0.2790697674418605</v>
+      </c>
+      <c r="W58" t="n">
+        <v>0.3906976744186046</v>
       </c>
     </row>
     <row r="59">
@@ -4577,19 +5293,19 @@
         <v>28.10494928575288</v>
       </c>
       <c r="J59" t="n">
-        <v>652.0106594184889</v>
+        <v>652.0106594184892</v>
       </c>
       <c r="K59" t="n">
-        <v>89.66979860087986</v>
+        <v>89.66979860088009</v>
       </c>
       <c r="L59" t="n">
-        <v>44.9912430763705</v>
+        <v>44.99124307637077</v>
       </c>
       <c r="M59" t="n">
-        <v>7.27124036846104</v>
+        <v>7.271240368461025</v>
       </c>
       <c r="N59" t="n">
-        <v>1.99305003528508</v>
+        <v>1.993050035285074</v>
       </c>
       <c r="O59" t="n">
         <v>16687718.71439746</v>
@@ -4606,6 +5322,18 @@
       <c r="S59" t="n">
         <v>5.184538161828589</v>
       </c>
+      <c r="T59" t="n">
+        <v>13368.40892985356</v>
+      </c>
+      <c r="U59" t="n">
+        <v>0.2706422018348624</v>
+      </c>
+      <c r="V59" t="n">
+        <v>0.2018348623853211</v>
+      </c>
+      <c r="W59" t="n">
+        <v>0.5275229357798165</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4648,19 +5376,19 @@
         <v>15.71170342029631</v>
       </c>
       <c r="J60" t="n">
-        <v>95.28225257504351</v>
+        <v>95.28225257504354</v>
       </c>
       <c r="K60" t="n">
-        <v>91.09311272535246</v>
+        <v>91.09311272535248</v>
       </c>
       <c r="L60" t="n">
-        <v>59.79211639749262</v>
+        <v>59.79211639749259</v>
       </c>
       <c r="M60" t="n">
         <v>1.045987448714387</v>
       </c>
       <c r="N60" t="n">
-        <v>1.523497046329212</v>
+        <v>1.523497046329213</v>
       </c>
       <c r="O60" t="n">
         <v>4101127.639690117</v>
@@ -4677,6 +5405,18 @@
       <c r="S60" t="n">
         <v>1.028092721960671</v>
       </c>
+      <c r="T60" t="n">
+        <v>8874.201805923758</v>
+      </c>
+      <c r="U60" t="n">
+        <v>0.1359223300970874</v>
+      </c>
+      <c r="V60" t="n">
+        <v>0.3203883495145631</v>
+      </c>
+      <c r="W60" t="n">
+        <v>0.5436893203883495</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4719,19 +5459,19 @@
         <v>28.00177256060446</v>
       </c>
       <c r="J61" t="n">
-        <v>430.8475572803292</v>
+        <v>430.8475572803289</v>
       </c>
       <c r="K61" t="n">
-        <v>198.2362130181201</v>
+        <v>198.23621301812</v>
       </c>
       <c r="L61" t="n">
-        <v>153.9488339982464</v>
+        <v>153.9488339982467</v>
       </c>
       <c r="M61" t="n">
-        <v>2.173404902770953</v>
+        <v>2.173404902770952</v>
       </c>
       <c r="N61" t="n">
-        <v>1.287675962653787</v>
+        <v>1.287675962653785</v>
       </c>
       <c r="O61" t="n">
         <v>32623760.18839955</v>
@@ -4748,6 +5488,18 @@
       <c r="S61" t="n">
         <v>1.652859362502283</v>
       </c>
+      <c r="T61" t="n">
+        <v>32302.86091526767</v>
+      </c>
+      <c r="U61" t="n">
+        <v>0.1774193548387097</v>
+      </c>
+      <c r="V61" t="n">
+        <v>0.2379032258064516</v>
+      </c>
+      <c r="W61" t="n">
+        <v>0.5846774193548387</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4790,19 +5542,19 @@
         <v>24.65643963677616</v>
       </c>
       <c r="J62" t="n">
-        <v>453.2664543618741</v>
+        <v>453.2664543618747</v>
       </c>
       <c r="K62" t="n">
         <v>101.2285305842539</v>
       </c>
       <c r="L62" t="n">
-        <v>50.21882732953713</v>
+        <v>50.21882732953709</v>
       </c>
       <c r="M62" t="n">
-        <v>4.477655180271676</v>
+        <v>4.477655180271681</v>
       </c>
       <c r="N62" t="n">
-        <v>2.015748594048002</v>
+        <v>2.015748594048004</v>
       </c>
       <c r="O62" t="n">
         <v>14594397.00831384</v>
@@ -4819,6 +5571,18 @@
       <c r="S62" t="n">
         <v>3.33560353137076</v>
       </c>
+      <c r="T62" t="n">
+        <v>15562.74125693551</v>
+      </c>
+      <c r="U62" t="n">
+        <v>0.2377049180327869</v>
+      </c>
+      <c r="V62" t="n">
+        <v>0.2254098360655738</v>
+      </c>
+      <c r="W62" t="n">
+        <v>0.5368852459016393</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4864,13 +5628,13 @@
         <v>217.5532425777894</v>
       </c>
       <c r="K63" t="n">
-        <v>60.62239192679314</v>
+        <v>60.62239192679309</v>
       </c>
       <c r="L63" t="n">
-        <v>54.34480635706274</v>
+        <v>54.34480635706267</v>
       </c>
       <c r="M63" t="n">
-        <v>3.588661477437314</v>
+        <v>3.588661477437317</v>
       </c>
       <c r="N63" t="n">
         <v>1.115513992790492</v>
@@ -4882,7 +5646,7 @@
         <v>3236049.205260403</v>
       </c>
       <c r="Q63" t="n">
-        <v>1375291.202761045</v>
+        <v>1375291.202761044</v>
       </c>
       <c r="R63" t="n">
         <v>1.028490867891062</v>
@@ -4890,6 +5654,18 @@
       <c r="S63" t="n">
         <v>2.35299200544851</v>
       </c>
+      <c r="T63" t="n">
+        <v>9081.494368917969</v>
+      </c>
+      <c r="U63" t="n">
+        <v>0.2155172413793103</v>
+      </c>
+      <c r="V63" t="n">
+        <v>0.2068965517241379</v>
+      </c>
+      <c r="W63" t="n">
+        <v>0.5775862068965517</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4932,22 +5708,22 @@
         <v>22.10591258533092</v>
       </c>
       <c r="J64" t="n">
-        <v>310.5016552702392</v>
+        <v>310.5016552702396</v>
       </c>
       <c r="K64" t="n">
-        <v>122.7800163055157</v>
+        <v>122.7800163055158</v>
       </c>
       <c r="L64" t="n">
-        <v>56.17019984677442</v>
+        <v>56.17019984677444</v>
       </c>
       <c r="M64" t="n">
-        <v>2.528926649574734</v>
+        <v>2.528926649574737</v>
       </c>
       <c r="N64" t="n">
         <v>2.185856853642054</v>
       </c>
       <c r="O64" t="n">
-        <v>10629593.27128405</v>
+        <v>10629593.27128404</v>
       </c>
       <c r="P64" t="n">
         <v>8968013.088267274</v>
@@ -4956,11 +5732,23 @@
         <v>4390311.503570621</v>
       </c>
       <c r="R64" t="n">
-        <v>1.185278518960972</v>
+        <v>1.185278518960971</v>
       </c>
       <c r="S64" t="n">
         <v>2.042682639027693</v>
       </c>
+      <c r="T64" t="n">
+        <v>14196.92286387182</v>
+      </c>
+      <c r="U64" t="n">
+        <v>0.2899159663865546</v>
+      </c>
+      <c r="V64" t="n">
+        <v>0.1848739495798319</v>
+      </c>
+      <c r="W64" t="n">
+        <v>0.5252100840336135</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5003,19 +5791,19 @@
         <v>29.79294036319115</v>
       </c>
       <c r="J65" t="n">
-        <v>541.0440796999432</v>
+        <v>541.0440796999435</v>
       </c>
       <c r="K65" t="n">
-        <v>224.4929624124694</v>
+        <v>224.4929624124701</v>
       </c>
       <c r="L65" t="n">
-        <v>116.3995137375663</v>
+        <v>116.3995137375664</v>
       </c>
       <c r="M65" t="n">
-        <v>2.410071451174769</v>
+        <v>2.410071451174764</v>
       </c>
       <c r="N65" t="n">
-        <v>1.928641754626313</v>
+        <v>1.928641754626316</v>
       </c>
       <c r="O65" t="n">
         <v>31193365.4711573</v>
@@ -5032,6 +5820,18 @@
       <c r="S65" t="n">
         <v>1.932369445294188</v>
       </c>
+      <c r="T65" t="n">
+        <v>31053.68862393996</v>
+      </c>
+      <c r="U65" t="n">
+        <v>0.2475</v>
+      </c>
+      <c r="V65" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="W65" t="n">
+        <v>0.5875</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5074,19 +5874,19 @@
         <v>29.14783405607515</v>
       </c>
       <c r="J66" t="n">
-        <v>513.5996852369491</v>
+        <v>513.5996852369485</v>
       </c>
       <c r="K66" t="n">
-        <v>291.4809983425544</v>
+        <v>291.4809983425542</v>
       </c>
       <c r="L66" t="n">
-        <v>44.63574234312483</v>
+        <v>44.63574234312491</v>
       </c>
       <c r="M66" t="n">
         <v>1.762034877598972</v>
       </c>
       <c r="N66" t="n">
-        <v>6.530215093139383</v>
+        <v>6.530215093139367</v>
       </c>
       <c r="O66" t="n">
         <v>17761424.63579462</v>
@@ -5103,6 +5903,18 @@
       <c r="S66" t="n">
         <v>1.662016485346259</v>
       </c>
+      <c r="T66" t="n">
+        <v>15530.25400815421</v>
+      </c>
+      <c r="U66" t="n">
+        <v>0.3051643192488263</v>
+      </c>
+      <c r="V66" t="n">
+        <v>0.1408450704225352</v>
+      </c>
+      <c r="W66" t="n">
+        <v>0.5539906103286385</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5145,34 +5957,46 @@
         <v>19.97174319614876</v>
       </c>
       <c r="J67" t="n">
-        <v>302.2783846918794</v>
+        <v>302.2783846918797</v>
       </c>
       <c r="K67" t="n">
-        <v>55.17654406826379</v>
+        <v>55.17654406826392</v>
       </c>
       <c r="L67" t="n">
         <v>38.70295853889188</v>
       </c>
       <c r="M67" t="n">
-        <v>5.478385603815709</v>
+        <v>5.478385603815701</v>
       </c>
       <c r="N67" t="n">
-        <v>1.425641505230612</v>
+        <v>1.425641505230615</v>
       </c>
       <c r="O67" t="n">
-        <v>6399895.485052345</v>
+        <v>6399895.485052346</v>
       </c>
       <c r="P67" t="n">
         <v>6107968.647797012</v>
       </c>
       <c r="Q67" t="n">
-        <v>1673531.492246803</v>
+        <v>1673531.492246802</v>
       </c>
       <c r="R67" t="n">
         <v>1.047794423005204</v>
       </c>
       <c r="S67" t="n">
-        <v>3.649748257558481</v>
+        <v>3.649748257558483</v>
+      </c>
+      <c r="T67" t="n">
+        <v>9955.657011291289</v>
+      </c>
+      <c r="U67" t="n">
+        <v>0.3728813559322034</v>
+      </c>
+      <c r="V67" t="n">
+        <v>0.1412429378531073</v>
+      </c>
+      <c r="W67" t="n">
+        <v>0.4858757062146893</v>
       </c>
     </row>
     <row r="68">
@@ -5216,19 +6040,19 @@
         <v>22.85157079258115</v>
       </c>
       <c r="J68" t="n">
-        <v>277.3330387570114</v>
+        <v>277.3330387570111</v>
       </c>
       <c r="K68" t="n">
-        <v>167.3979710824163</v>
+        <v>167.3979710824161</v>
       </c>
       <c r="L68" t="n">
-        <v>74.67300296935787</v>
+        <v>74.67300296935822</v>
       </c>
       <c r="M68" t="n">
         <v>1.656728794045359</v>
       </c>
       <c r="N68" t="n">
-        <v>2.241746875388261</v>
+        <v>2.241746875388248</v>
       </c>
       <c r="O68" t="n">
         <v>16485987.15732341</v>
@@ -5237,13 +6061,25 @@
         <v>13054172.47394027</v>
       </c>
       <c r="Q68" t="n">
-        <v>8952786.540309219</v>
+        <v>8952786.540309228</v>
       </c>
       <c r="R68" t="n">
         <v>1.262890251391575</v>
       </c>
       <c r="S68" t="n">
-        <v>1.458112780324303</v>
+        <v>1.458112780324301</v>
+      </c>
+      <c r="T68" t="n">
+        <v>19404.25804932194</v>
+      </c>
+      <c r="U68" t="n">
+        <v>0.3468208092485549</v>
+      </c>
+      <c r="V68" t="n">
+        <v>0.2630057803468208</v>
+      </c>
+      <c r="W68" t="n">
+        <v>0.3901734104046243</v>
       </c>
     </row>
     <row r="69">
@@ -5290,22 +6126,22 @@
         <v>256.0287304080996</v>
       </c>
       <c r="K69" t="n">
-        <v>83.95547371371968</v>
+        <v>83.95547371371984</v>
       </c>
       <c r="L69" t="n">
-        <v>42.43829781800725</v>
+        <v>42.43829781800746</v>
       </c>
       <c r="M69" t="n">
-        <v>3.049577580624864</v>
+        <v>3.049577580624858</v>
       </c>
       <c r="N69" t="n">
-        <v>1.978295031383093</v>
+        <v>1.978295031383086</v>
       </c>
       <c r="O69" t="n">
         <v>5573015.479494516</v>
       </c>
       <c r="P69" t="n">
-        <v>4891024.393152248</v>
+        <v>4891024.393152246</v>
       </c>
       <c r="Q69" t="n">
         <v>2068031.94393085</v>
@@ -5316,6 +6152,18 @@
       <c r="S69" t="n">
         <v>2.365062303561686</v>
       </c>
+      <c r="T69" t="n">
+        <v>9600.901634393274</v>
+      </c>
+      <c r="U69" t="n">
+        <v>0.4150943396226415</v>
+      </c>
+      <c r="V69" t="n">
+        <v>0.1761006289308176</v>
+      </c>
+      <c r="W69" t="n">
+        <v>0.4088050314465409</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5358,19 +6206,19 @@
         <v>22.86657816384182</v>
       </c>
       <c r="J70" t="n">
-        <v>398.8677503319433</v>
+        <v>398.867750331943</v>
       </c>
       <c r="K70" t="n">
-        <v>79.84017969925321</v>
+        <v>79.84017969925318</v>
       </c>
       <c r="L70" t="n">
-        <v>46.23460498245312</v>
+        <v>46.23460498245321</v>
       </c>
       <c r="M70" t="n">
-        <v>4.995827311942712</v>
+        <v>4.99582731194271</v>
       </c>
       <c r="N70" t="n">
-        <v>1.726848963661613</v>
+        <v>1.726848963661609</v>
       </c>
       <c r="O70" t="n">
         <v>8231977.956016028</v>
@@ -5387,6 +6235,18 @@
       <c r="S70" t="n">
         <v>3.49438544058357</v>
       </c>
+      <c r="T70" t="n">
+        <v>10694.88552730892</v>
+      </c>
+      <c r="U70" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="V70" t="n">
+        <v>0.1726190476190476</v>
+      </c>
+      <c r="W70" t="n">
+        <v>0.4523809523809524</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5429,19 +6289,19 @@
         <v>23.31354361192112</v>
       </c>
       <c r="J71" t="n">
-        <v>434.546746019599</v>
+        <v>434.5467460195982</v>
       </c>
       <c r="K71" t="n">
-        <v>55.41610952953412</v>
+        <v>55.416109529534</v>
       </c>
       <c r="L71" t="n">
-        <v>52.09567145614087</v>
+        <v>52.0956714561408</v>
       </c>
       <c r="M71" t="n">
-        <v>7.84152387651837</v>
+        <v>7.841523876518373</v>
       </c>
       <c r="N71" t="n">
-        <v>1.063737312152483</v>
+        <v>1.063737312152482</v>
       </c>
       <c r="O71" t="n">
         <v>10576189.94183022</v>
@@ -5450,13 +6310,25 @@
         <v>10504087.74529458</v>
       </c>
       <c r="Q71" t="n">
-        <v>2310415.416892178</v>
+        <v>2310415.41689218</v>
       </c>
       <c r="R71" t="n">
         <v>1.006864203563792</v>
       </c>
       <c r="S71" t="n">
-        <v>4.546406532996564</v>
+        <v>4.546406532996561</v>
+      </c>
+      <c r="T71" t="n">
+        <v>11955.39615111158</v>
+      </c>
+      <c r="U71" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="V71" t="n">
+        <v>0.1714285714285714</v>
+      </c>
+      <c r="W71" t="n">
+        <v>0.5428571428571428</v>
       </c>
     </row>
     <row r="72">
@@ -5500,28 +6372,28 @@
         <v>54.15486713045508</v>
       </c>
       <c r="J72" t="n">
-        <v>1193.115832962802</v>
+        <v>1193.115832962803</v>
       </c>
       <c r="K72" t="n">
         <v>1001.699460963759</v>
       </c>
       <c r="L72" t="n">
-        <v>727.7128649621889</v>
+        <v>727.7128649621899</v>
       </c>
       <c r="M72" t="n">
-        <v>1.191091619251623</v>
+        <v>1.191091619251624</v>
       </c>
       <c r="N72" t="n">
-        <v>1.37650371347469</v>
+        <v>1.376503713474688</v>
       </c>
       <c r="O72" t="n">
         <v>183063744.4046845</v>
       </c>
       <c r="P72" t="n">
-        <v>160221317.1822739</v>
+        <v>160221317.182274</v>
       </c>
       <c r="Q72" t="n">
-        <v>144336386.7378148</v>
+        <v>144336386.7378149</v>
       </c>
       <c r="R72" t="n">
         <v>1.142567965512505</v>
@@ -5529,6 +6401,18 @@
       <c r="S72" t="n">
         <v>1.110054926574502</v>
       </c>
+      <c r="T72" t="n">
+        <v>97502.40103155182</v>
+      </c>
+      <c r="U72" t="n">
+        <v>0.09194097616345062</v>
+      </c>
+      <c r="V72" t="n">
+        <v>0.03064699205448354</v>
+      </c>
+      <c r="W72" t="n">
+        <v>0.8774120317820658</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5571,19 +6455,19 @@
         <v>16.28960679610518</v>
       </c>
       <c r="J73" t="n">
-        <v>136.039129682857</v>
+        <v>136.0391296828571</v>
       </c>
       <c r="K73" t="n">
-        <v>74.89472676165826</v>
+        <v>74.89472676165838</v>
       </c>
       <c r="L73" t="n">
-        <v>54.14273635670478</v>
+        <v>54.14273635670492</v>
       </c>
       <c r="M73" t="n">
-        <v>1.81640464642834</v>
+        <v>1.816404646428338</v>
       </c>
       <c r="N73" t="n">
-        <v>1.383282999740438</v>
+        <v>1.383282999740437</v>
       </c>
       <c r="O73" t="n">
         <v>4307638.771641318</v>
@@ -5600,6 +6484,18 @@
       <c r="S73" t="n">
         <v>1.485962444029307</v>
       </c>
+      <c r="T73" t="n">
+        <v>10005.9854351411</v>
+      </c>
+      <c r="U73" t="n">
+        <v>0.2617801047120419</v>
+      </c>
+      <c r="V73" t="n">
+        <v>0.225130890052356</v>
+      </c>
+      <c r="W73" t="n">
+        <v>0.5130890052356021</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5642,19 +6538,19 @@
         <v>25.46884714093742</v>
       </c>
       <c r="J74" t="n">
-        <v>521.8886874447543</v>
+        <v>521.8886874447549</v>
       </c>
       <c r="K74" t="n">
-        <v>72.35949362736272</v>
+        <v>72.35949362736268</v>
       </c>
       <c r="L74" t="n">
-        <v>49.36016401697255</v>
+        <v>49.36016401697266</v>
       </c>
       <c r="M74" t="n">
-        <v>7.212442504536851</v>
+        <v>7.212442504536862</v>
       </c>
       <c r="N74" t="n">
-        <v>1.465949213671207</v>
+        <v>1.465949213671203</v>
       </c>
       <c r="O74" t="n">
         <v>10277040.97476912</v>
@@ -5671,6 +6567,18 @@
       <c r="S74" t="n">
         <v>4.732365610337142</v>
       </c>
+      <c r="T74" t="n">
+        <v>10775.14531796634</v>
+      </c>
+      <c r="U74" t="n">
+        <v>0.281437125748503</v>
+      </c>
+      <c r="V74" t="n">
+        <v>0.1736526946107785</v>
+      </c>
+      <c r="W74" t="n">
+        <v>0.5449101796407185</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5713,19 +6621,19 @@
         <v>18.98296067271316</v>
       </c>
       <c r="J75" t="n">
-        <v>250.1316060365307</v>
+        <v>250.1316060365305</v>
       </c>
       <c r="K75" t="n">
-        <v>63.60321072106348</v>
+        <v>63.60321072106349</v>
       </c>
       <c r="L75" t="n">
-        <v>45.25159285738057</v>
+        <v>45.25159285738061</v>
       </c>
       <c r="M75" t="n">
-        <v>3.932688353320732</v>
+        <v>3.932688353320729</v>
       </c>
       <c r="N75" t="n">
-        <v>1.405546340026564</v>
+        <v>1.405546340026563</v>
       </c>
       <c r="O75" t="n">
         <v>5194831.245366923</v>
@@ -5742,6 +6650,18 @@
       <c r="S75" t="n">
         <v>2.723173109721641</v>
       </c>
+      <c r="T75" t="n">
+        <v>9339.519881634018</v>
+      </c>
+      <c r="U75" t="n">
+        <v>0.3963414634146342</v>
+      </c>
+      <c r="V75" t="n">
+        <v>0.1768292682926829</v>
+      </c>
+      <c r="W75" t="n">
+        <v>0.4268292682926829</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5784,25 +6704,25 @@
         <v>29.94417168731466</v>
       </c>
       <c r="J76" t="n">
-        <v>435.6630354087017</v>
+        <v>435.6630354087001</v>
       </c>
       <c r="K76" t="n">
         <v>387.4038372199308</v>
       </c>
       <c r="L76" t="n">
-        <v>74.24419129751203</v>
+        <v>74.24419129751186</v>
       </c>
       <c r="M76" t="n">
-        <v>1.124570780029145</v>
+        <v>1.124570780029141</v>
       </c>
       <c r="N76" t="n">
-        <v>5.217968307682448</v>
+        <v>5.217968307682461</v>
       </c>
       <c r="O76" t="n">
-        <v>48924487.17116658</v>
+        <v>48924487.17116657</v>
       </c>
       <c r="P76" t="n">
-        <v>30322727.08534741</v>
+        <v>30322727.0853474</v>
       </c>
       <c r="Q76" t="n">
         <v>27460955.35541772</v>
@@ -5813,6 +6733,18 @@
       <c r="S76" t="n">
         <v>1.104212387839052</v>
       </c>
+      <c r="T76" t="n">
+        <v>25144.65652929292</v>
+      </c>
+      <c r="U76" t="n">
+        <v>0.4577702702702703</v>
+      </c>
+      <c r="V76" t="n">
+        <v>0.1790540540540541</v>
+      </c>
+      <c r="W76" t="n">
+        <v>0.3631756756756757</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5855,7 +6787,7 @@
         <v>22.88678799452688</v>
       </c>
       <c r="J77" t="n">
-        <v>289.0215660571018</v>
+        <v>289.0215660571015</v>
       </c>
       <c r="K77" t="n">
         <v>131.8633861355019</v>
@@ -5864,7 +6796,7 @@
         <v>103.6837219565705</v>
       </c>
       <c r="M77" t="n">
-        <v>2.191825756393859</v>
+        <v>2.191825756393856</v>
       </c>
       <c r="N77" t="n">
         <v>1.271784843822783</v>
@@ -5884,6 +6816,18 @@
       <c r="S77" t="n">
         <v>1.663816572053927</v>
       </c>
+      <c r="T77" t="n">
+        <v>19129.17745584282</v>
+      </c>
+      <c r="U77" t="n">
+        <v>0.5790816326530612</v>
+      </c>
+      <c r="V77" t="n">
+        <v>0.07142857142857142</v>
+      </c>
+      <c r="W77" t="n">
+        <v>0.3494897959183674</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5926,19 +6870,19 @@
         <v>20.05156727857752</v>
       </c>
       <c r="J78" t="n">
-        <v>365.0650463190738</v>
+        <v>365.0650463190735</v>
       </c>
       <c r="K78" t="n">
         <v>26.38310595604296</v>
       </c>
       <c r="L78" t="n">
-        <v>9.679078078446759</v>
+        <v>9.679078078446894</v>
       </c>
       <c r="M78" t="n">
-        <v>13.8370761549952</v>
+        <v>13.83707615499519</v>
       </c>
       <c r="N78" t="n">
-        <v>2.725787078295453</v>
+        <v>2.725787078295415</v>
       </c>
       <c r="O78" t="n">
         <v>2150493.793621778</v>
@@ -5947,13 +6891,25 @@
         <v>2057227.674662992</v>
       </c>
       <c r="Q78" t="n">
-        <v>197105.4772261902</v>
+        <v>197105.4772261896</v>
       </c>
       <c r="R78" t="n">
         <v>1.045335827486408</v>
       </c>
       <c r="S78" t="n">
-        <v>10.43719182040893</v>
+        <v>10.43719182040897</v>
+      </c>
+      <c r="T78" t="n">
+        <v>5445.388003466757</v>
+      </c>
+      <c r="U78" t="n">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="V78" t="n">
+        <v>0</v>
+      </c>
+      <c r="W78" t="n">
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="79">
@@ -5997,16 +6953,16 @@
         <v>13.37163211023283</v>
       </c>
       <c r="J79" t="n">
-        <v>82.74873733913223</v>
+        <v>82.74873733913216</v>
       </c>
       <c r="K79" t="n">
-        <v>61.75316867051429</v>
+        <v>61.75316867051428</v>
       </c>
       <c r="L79" t="n">
         <v>33.97112894364543</v>
       </c>
       <c r="M79" t="n">
-        <v>1.339991762700314</v>
+        <v>1.339991762700313</v>
       </c>
       <c r="N79" t="n">
         <v>1.817813260576543</v>
@@ -6026,6 +6982,18 @@
       <c r="S79" t="n">
         <v>1.223013014477382</v>
       </c>
+      <c r="T79" t="n">
+        <v>6557.61834591064</v>
+      </c>
+      <c r="U79" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="V79" t="n">
+        <v>0.216</v>
+      </c>
+      <c r="W79" t="n">
+        <v>0.336</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6068,19 +7036,19 @@
         <v>11.23263894292782</v>
       </c>
       <c r="J80" t="n">
-        <v>62.01416381394563</v>
+        <v>62.01416381394561</v>
       </c>
       <c r="K80" t="n">
-        <v>41.05432154998153</v>
+        <v>41.05432154998154</v>
       </c>
       <c r="L80" t="n">
-        <v>23.01760901492504</v>
+        <v>23.01760901492502</v>
       </c>
       <c r="M80" t="n">
         <v>1.510539243437419</v>
       </c>
       <c r="N80" t="n">
-        <v>1.783604957550594</v>
+        <v>1.783604957550595</v>
       </c>
       <c r="O80" t="n">
         <v>648132.2813429361</v>
@@ -6097,6 +7065,18 @@
       <c r="S80" t="n">
         <v>1.330239340318172</v>
       </c>
+      <c r="T80" t="n">
+        <v>4688.756053298779</v>
+      </c>
+      <c r="U80" t="n">
+        <v>0.3934426229508197</v>
+      </c>
+      <c r="V80" t="n">
+        <v>0.2786885245901639</v>
+      </c>
+      <c r="W80" t="n">
+        <v>0.3278688524590164</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6139,34 +7119,46 @@
         <v>48.42584107779204</v>
       </c>
       <c r="J81" t="n">
-        <v>1978.228843556296</v>
+        <v>1978.228843556298</v>
       </c>
       <c r="K81" t="n">
-        <v>233.7544614394139</v>
+        <v>233.7544614394137</v>
       </c>
       <c r="L81" t="n">
-        <v>129.359224884891</v>
+        <v>129.3592248848915</v>
       </c>
       <c r="M81" t="n">
-        <v>8.462849570334413</v>
+        <v>8.462849570334427</v>
       </c>
       <c r="N81" t="n">
-        <v>1.807018105182819</v>
+        <v>1.807018105182811</v>
       </c>
       <c r="O81" t="n">
-        <v>97443475.94884828</v>
+        <v>97443475.94884831</v>
       </c>
       <c r="P81" t="n">
-        <v>92858099.88929792</v>
+        <v>92858099.8892979</v>
       </c>
       <c r="Q81" t="n">
-        <v>16064084.54712701</v>
+        <v>16064084.54712704</v>
       </c>
       <c r="R81" t="n">
-        <v>1.049380464009245</v>
+        <v>1.049380464009246</v>
       </c>
       <c r="S81" t="n">
-        <v>5.780478782770425</v>
+        <v>5.780478782770413</v>
+      </c>
+      <c r="T81" t="n">
+        <v>35165.78581850311</v>
+      </c>
+      <c r="U81" t="n">
+        <v>0.5857461024498887</v>
+      </c>
+      <c r="V81" t="n">
+        <v>0.04231625835189309</v>
+      </c>
+      <c r="W81" t="n">
+        <v>0.3719376391982183</v>
       </c>
     </row>
     <row r="82">
@@ -6210,34 +7202,46 @@
         <v>48.62167273522643</v>
       </c>
       <c r="J82" t="n">
-        <v>2314.660217227289</v>
+        <v>2314.660217227287</v>
       </c>
       <c r="K82" t="n">
-        <v>28.12528315415419</v>
+        <v>28.1252831541555</v>
       </c>
       <c r="L82" t="n">
-        <v>24.72116052570183</v>
+        <v>24.72116052570177</v>
       </c>
       <c r="M82" t="n">
-        <v>82.2982013919887</v>
+        <v>82.29820139198482</v>
       </c>
       <c r="N82" t="n">
-        <v>1.137700761455483</v>
+        <v>1.137700761455538</v>
       </c>
       <c r="O82" t="n">
-        <v>53795383.11348493</v>
+        <v>53795383.11348492</v>
       </c>
       <c r="P82" t="n">
         <v>53720200.92444175</v>
       </c>
       <c r="Q82" t="n">
-        <v>1219959.326975638</v>
+        <v>1219959.326975642</v>
       </c>
       <c r="R82" t="n">
         <v>1.001399514293495</v>
       </c>
       <c r="S82" t="n">
-        <v>44.03441962087192</v>
+        <v>44.03441962087179</v>
+      </c>
+      <c r="T82" t="n">
+        <v>17433.86836999504</v>
+      </c>
+      <c r="U82" t="n">
+        <v>0.9517543859649122</v>
+      </c>
+      <c r="V82" t="n">
+        <v>0</v>
+      </c>
+      <c r="W82" t="n">
+        <v>0.04824561403508772</v>
       </c>
     </row>
     <row r="83">
@@ -6284,16 +7288,16 @@
         <v>73.05924276329493</v>
       </c>
       <c r="K83" t="n">
-        <v>44.64869983598494</v>
+        <v>44.64869983598491</v>
       </c>
       <c r="L83" t="n">
-        <v>34.40822721925166</v>
+        <v>34.40822721925169</v>
       </c>
       <c r="M83" t="n">
-        <v>1.636312883279354</v>
+        <v>1.636312883279355</v>
       </c>
       <c r="N83" t="n">
-        <v>1.297616978389508</v>
+        <v>1.297616978389506</v>
       </c>
       <c r="O83" t="n">
         <v>1248668.754516886</v>
@@ -6302,13 +7306,25 @@
         <v>1141191.935038354</v>
       </c>
       <c r="Q83" t="n">
-        <v>840674.6523297314</v>
+        <v>840674.6523297315</v>
       </c>
       <c r="R83" t="n">
-        <v>1.094179441843777</v>
+        <v>1.094179441843776</v>
       </c>
       <c r="S83" t="n">
         <v>1.357471563910973</v>
+      </c>
+      <c r="T83" t="n">
+        <v>5401.894134831939</v>
+      </c>
+      <c r="U83" t="n">
+        <v>0.462962962962963</v>
+      </c>
+      <c r="V83" t="n">
+        <v>0.1851851851851852</v>
+      </c>
+      <c r="W83" t="n">
+        <v>0.3518518518518519</v>
       </c>
     </row>
   </sheetData>

</xml_diff>